<commit_message>
docs: add cross-browser evidence and update counts to 57 runs
Full suite reports for Chrome 153 and Firefox 156, both 56 run and 0 failed. The full suite
is committed rather than smoke because CI only runs the smoke suite, so these are the only
evidence that the regression-only tests pass.

TC_NEG_012 now runs once per route, so the suite is 57 runs (56 plus the excluded known
defect). README, framework notes and the test case document updated to match, including the
reworked TC_NEG_012 row and finding F-14 on the defect Firefox exposed in the test.
</commit_message>
<xml_diff>
--- a/MBio_Test_Cases.xlsx
+++ b/MBio_Test_Cases.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1839" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2466" uniqueCount="361">
   <si>
     <t>TC_NAV_001</t>
   </si>
@@ -1216,6 +1216,43 @@
   </si>
   <si>
     <t>Heading capitalisation is not stable. The Blog page heading was read as 'Blog and News' at 17:40 and 'Blog and news' at 17:51 on 17 Sep 2026, in two runs 11 minutes apart. Page headings are therefore compared with AssertUtils.verifyEqualsIgnoreCase - the words must match exactly, only upper / lower case is tolerated.</t>
+  </si>
+  <si>
+    <t>Verify a protected route redirects a guest to the login page (data-driven, one run per route)</t>
+  </si>
+  <si>
+    <t>Routes: /trade, /explore, /wallet - one test run each</t>
+  </si>
+  <si>
+    <t>1. Open trade.mb.io{route} as a guest
+2. Wait until the URL carries the full next parameter for that route
+3. Read the login URL</t>
+  </si>
+  <si>
+    <t>1. The route redirects to the login page
+2. The login URL carries next={route} so the user returns after logging in
+3. No credentials are entered</t>
+  </si>
+  <si>
+    <t>InvalidRouteTest.verifyProtectedRouteRedirectsGuestToLogin</t>
+  </si>
+  <si>
+    <t>One run per route so each starts in a fresh browser. The routes were originally checked in a loop in one test; every route after the first then began on the previous route's login page, and the wait for '/login' was already satisfied, so the check read the old URL. Firefox exposed this on /wallet - see finding F-14. Only the first path segment is used: a deeper URL like /wallet/spot/overview sends the guest to /login?next=/wallet.</t>
+  </si>
+  <si>
+    <t>F-14</t>
+  </si>
+  <si>
+    <t>Checking several routes in one test hid a defect in the test itself. After the first route the browser was already on a login page, so waiting for '/login' was satisfied at once and the check read the previous route's URL. Chrome finished navigating quickly enough to mask it; Firefox did not. TC_NEG_012 now runs once per route, in a fresh browser, and waits for the full next parameter rather than just '/login'.</t>
+  </si>
+  <si>
+    <t>2026-09-18 - testng.xml - 56 tests run, 0 failures - on Chrome 153 and on Firefox 156. 1 further test (TC_NEG_002-KI) is excluded by the 'known-issue' group and fails on purpose.</t>
+  </si>
+  <si>
+    <t>2026-09-18</t>
+  </si>
+  <si>
+    <t>Chrome 153 and Firefox 156, 1920x1080. Both browsers run the same suite - see docs/sample-reports/</t>
   </si>
 </sst>
 </file>
@@ -1299,7 +1336,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1326,6 +1363,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+      <alignment wrapText="true" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
       <alignment wrapText="true" vertical="top"/>
@@ -1772,11 +1812,8 @@
           <t>Default browser / viewport</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <v>Chrome (latest) 1920x1080. The same suite also runs on Firefox in CI - see docs/sample-reports/</v>
-        <is>
-          <t>Chrome latest · 1920x1080 (desktop) · 390x844 (mobile)</t>
-        </is>
+      <c r="B7" t="s" s="3">
+        <v>360</v>
       </c>
     </row>
     <row r="8">
@@ -1797,11 +1834,8 @@
           <t>Date</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <v>2026-09-17</v>
-        <is>
-          <t>2026-09-14</t>
-        </is>
+      <c r="B9" t="s" s="3">
+        <v>359</v>
       </c>
     </row>
     <row r="10">
@@ -1833,7 +1867,7 @@
         <v>345</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>346</v>
+        <v>358</v>
       </c>
     </row>
     <row r="14">
@@ -2116,1553 +2150,1553 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="15">
+      <c r="A2" t="s" s="16">
         <v>0</v>
       </c>
-      <c r="B2" t="s" s="15">
+      <c r="B2" t="s" s="16">
         <v>1</v>
       </c>
-      <c r="C2" t="s" s="15">
+      <c r="C2" t="s" s="16">
         <v>2</v>
       </c>
-      <c r="D2" t="s" s="15">
+      <c r="D2" t="s" s="16">
         <v>3</v>
       </c>
-      <c r="E2" t="s" s="15">
+      <c r="E2" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F2" t="s" s="15">
+      <c r="F2" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G2" t="s" s="15">
+      <c r="G2" t="s" s="16">
         <v>6</v>
       </c>
-      <c r="H2" t="s" s="15">
+      <c r="H2" t="s" s="16">
         <v>7</v>
       </c>
-      <c r="I2" t="s" s="15">
+      <c r="I2" t="s" s="16">
         <v>8</v>
       </c>
-      <c r="J2" t="s" s="15">
+      <c r="J2" t="s" s="16">
         <v>9</v>
       </c>
-      <c r="K2" t="s" s="15">
+      <c r="K2" t="s" s="16">
         <v>10</v>
       </c>
-      <c r="L2" t="s" s="15">
+      <c r="L2" t="s" s="16">
         <v>11</v>
       </c>
-      <c r="M2" t="s" s="15">
+      <c r="M2" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N2" t="s" s="15">
+      <c r="N2" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P2" t="s" s="15">
+      <c r="P2" t="s" s="16">
         <v>14</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="15">
+      <c r="A3" t="s" s="16">
         <v>15</v>
       </c>
-      <c r="B3" t="s" s="15">
+      <c r="B3" t="s" s="16">
         <v>1</v>
       </c>
-      <c r="C3" t="s" s="15">
+      <c r="C3" t="s" s="16">
         <v>16</v>
       </c>
-      <c r="D3" t="s" s="15">
+      <c r="D3" t="s" s="16">
         <v>17</v>
       </c>
-      <c r="E3" t="s" s="15">
+      <c r="E3" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F3" t="s" s="15">
+      <c r="F3" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G3" t="s" s="15">
+      <c r="G3" t="s" s="16">
         <v>18</v>
       </c>
-      <c r="H3" t="s" s="15">
+      <c r="H3" t="s" s="16">
         <v>19</v>
       </c>
-      <c r="I3" t="s" s="15">
+      <c r="I3" t="s" s="16">
         <v>20</v>
       </c>
-      <c r="J3" t="s" s="15">
+      <c r="J3" t="s" s="16">
         <v>21</v>
       </c>
-      <c r="K3" t="s" s="15">
+      <c r="K3" t="s" s="16">
         <v>22</v>
       </c>
-      <c r="L3" t="s" s="15">
+      <c r="L3" t="s" s="16">
         <v>23</v>
       </c>
-      <c r="M3" t="s" s="15">
+      <c r="M3" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N3" t="s" s="15">
+      <c r="N3" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P3" t="s" s="15">
+      <c r="P3" t="s" s="16">
         <v>347</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s" s="15">
+      <c r="A4" t="s" s="16">
         <v>25</v>
       </c>
-      <c r="B4" t="s" s="15">
+      <c r="B4" t="s" s="16">
         <v>1</v>
       </c>
-      <c r="C4" t="s" s="15">
+      <c r="C4" t="s" s="16">
         <v>16</v>
       </c>
-      <c r="D4" t="s" s="15">
+      <c r="D4" t="s" s="16">
         <v>26</v>
       </c>
-      <c r="E4" t="s" s="15">
+      <c r="E4" t="s" s="16">
         <v>27</v>
       </c>
-      <c r="F4" t="s" s="15">
+      <c r="F4" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G4" t="s" s="15">
+      <c r="G4" t="s" s="16">
         <v>18</v>
       </c>
-      <c r="H4" t="s" s="15">
+      <c r="H4" t="s" s="16">
         <v>28</v>
       </c>
-      <c r="I4" t="s" s="15">
+      <c r="I4" t="s" s="16">
         <v>29</v>
       </c>
-      <c r="J4" t="s" s="15">
+      <c r="J4" t="s" s="16">
         <v>30</v>
       </c>
-      <c r="K4" t="s" s="15">
+      <c r="K4" t="s" s="16">
         <v>31</v>
       </c>
-      <c r="L4" t="s" s="15">
+      <c r="L4" t="s" s="16">
         <v>32</v>
       </c>
-      <c r="M4" t="s" s="15">
+      <c r="M4" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N4" t="s" s="15">
+      <c r="N4" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P4" t="s" s="15">
+      <c r="P4" t="s" s="16">
         <v>33</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s" s="15">
+      <c r="A5" t="s" s="16">
         <v>34</v>
       </c>
-      <c r="B5" t="s" s="15">
+      <c r="B5" t="s" s="16">
         <v>1</v>
       </c>
-      <c r="C5" t="s" s="15">
+      <c r="C5" t="s" s="16">
         <v>16</v>
       </c>
-      <c r="D5" t="s" s="15">
+      <c r="D5" t="s" s="16">
         <v>35</v>
       </c>
-      <c r="E5" t="s" s="15">
+      <c r="E5" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F5" t="s" s="15">
+      <c r="F5" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G5" t="s" s="15">
+      <c r="G5" t="s" s="16">
         <v>18</v>
       </c>
-      <c r="H5" t="s" s="15">
+      <c r="H5" t="s" s="16">
         <v>36</v>
       </c>
-      <c r="I5" t="s" s="15">
+      <c r="I5" t="s" s="16">
         <v>37</v>
       </c>
-      <c r="J5" t="s" s="15">
+      <c r="J5" t="s" s="16">
         <v>38</v>
       </c>
-      <c r="K5" t="s" s="15">
+      <c r="K5" t="s" s="16">
         <v>10</v>
       </c>
-      <c r="L5" t="s" s="15">
+      <c r="L5" t="s" s="16">
         <v>39</v>
       </c>
-      <c r="M5" t="s" s="15">
+      <c r="M5" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N5" t="s" s="15">
+      <c r="N5" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P5" t="s" s="15">
+      <c r="P5" t="s" s="16">
         <v>40</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s" s="15">
+      <c r="A6" t="s" s="16">
         <v>41</v>
       </c>
-      <c r="B6" t="s" s="15">
+      <c r="B6" t="s" s="16">
         <v>1</v>
       </c>
-      <c r="C6" t="s" s="15">
+      <c r="C6" t="s" s="16">
         <v>42</v>
       </c>
-      <c r="D6" t="s" s="15">
+      <c r="D6" t="s" s="16">
         <v>43</v>
       </c>
-      <c r="E6" t="s" s="15">
+      <c r="E6" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F6" t="s" s="15">
+      <c r="F6" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G6" t="s" s="15">
+      <c r="G6" t="s" s="16">
         <v>44</v>
       </c>
-      <c r="H6" t="s" s="15">
+      <c r="H6" t="s" s="16">
         <v>45</v>
       </c>
-      <c r="I6" t="s" s="15">
+      <c r="I6" t="s" s="16">
         <v>46</v>
       </c>
-      <c r="J6" t="s" s="15">
+      <c r="J6" t="s" s="16">
         <v>47</v>
       </c>
-      <c r="K6" t="s" s="15">
+      <c r="K6" t="s" s="16">
         <v>22</v>
       </c>
-      <c r="L6" t="s" s="15">
+      <c r="L6" t="s" s="16">
         <v>48</v>
       </c>
-      <c r="M6" t="s" s="15">
+      <c r="M6" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N6" t="s" s="15">
+      <c r="N6" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P6" t="s" s="15">
+      <c r="P6" t="s" s="16">
         <v>49</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s" s="15">
+      <c r="A7" t="s" s="16">
         <v>50</v>
       </c>
-      <c r="B7" t="s" s="15">
+      <c r="B7" t="s" s="16">
         <v>1</v>
       </c>
-      <c r="C7" t="s" s="15">
+      <c r="C7" t="s" s="16">
         <v>16</v>
       </c>
-      <c r="D7" t="s" s="15">
+      <c r="D7" t="s" s="16">
         <v>51</v>
       </c>
-      <c r="E7" t="s" s="15">
+      <c r="E7" t="s" s="16">
         <v>27</v>
       </c>
-      <c r="F7" t="s" s="15">
+      <c r="F7" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G7" t="s" s="15">
+      <c r="G7" t="s" s="16">
         <v>18</v>
       </c>
-      <c r="H7" t="s" s="15">
+      <c r="H7" t="s" s="16">
         <v>52</v>
       </c>
-      <c r="I7" t="s" s="15">
+      <c r="I7" t="s" s="16">
         <v>53</v>
       </c>
-      <c r="J7" t="s" s="15">
+      <c r="J7" t="s" s="16">
         <v>54</v>
       </c>
-      <c r="K7" t="s" s="15">
+      <c r="K7" t="s" s="16">
         <v>31</v>
       </c>
-      <c r="L7" t="s" s="15">
+      <c r="L7" t="s" s="16">
         <v>55</v>
       </c>
-      <c r="M7" t="s" s="15">
+      <c r="M7" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N7" t="s" s="15">
+      <c r="N7" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P7" t="s" s="15">
+      <c r="P7" t="s" s="16">
         <v>13</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="s" s="15">
+      <c r="A8" t="s" s="16">
         <v>56</v>
       </c>
-      <c r="B8" t="s" s="15">
+      <c r="B8" t="s" s="16">
         <v>57</v>
       </c>
-      <c r="C8" t="s" s="15">
+      <c r="C8" t="s" s="16">
         <v>58</v>
       </c>
-      <c r="D8" t="s" s="15">
+      <c r="D8" t="s" s="16">
         <v>59</v>
       </c>
-      <c r="E8" t="s" s="15">
+      <c r="E8" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F8" t="s" s="15">
+      <c r="F8" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G8" t="s" s="15">
+      <c r="G8" t="s" s="16">
         <v>60</v>
       </c>
-      <c r="H8" t="s" s="15">
+      <c r="H8" t="s" s="16">
         <v>61</v>
       </c>
-      <c r="I8" t="s" s="15">
+      <c r="I8" t="s" s="16">
         <v>62</v>
       </c>
-      <c r="J8" t="s" s="15">
+      <c r="J8" t="s" s="16">
         <v>63</v>
       </c>
-      <c r="K8" t="s" s="15">
+      <c r="K8" t="s" s="16">
         <v>64</v>
       </c>
-      <c r="L8" t="s" s="15">
+      <c r="L8" t="s" s="16">
         <v>65</v>
       </c>
-      <c r="M8" t="s" s="15">
+      <c r="M8" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N8" t="s" s="15">
+      <c r="N8" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P8" t="s" s="15">
+      <c r="P8" t="s" s="16">
         <v>66</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="s" s="15">
+      <c r="A9" t="s" s="16">
         <v>67</v>
       </c>
-      <c r="B9" t="s" s="15">
+      <c r="B9" t="s" s="16">
         <v>57</v>
       </c>
-      <c r="C9" t="s" s="15">
+      <c r="C9" t="s" s="16">
         <v>58</v>
       </c>
-      <c r="D9" t="s" s="15">
+      <c r="D9" t="s" s="16">
         <v>68</v>
       </c>
-      <c r="E9" t="s" s="15">
+      <c r="E9" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F9" t="s" s="15">
+      <c r="F9" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G9" t="s" s="15">
+      <c r="G9" t="s" s="16">
         <v>69</v>
       </c>
-      <c r="H9" t="s" s="15">
+      <c r="H9" t="s" s="16">
         <v>70</v>
       </c>
-      <c r="I9" t="s" s="15">
+      <c r="I9" t="s" s="16">
         <v>71</v>
       </c>
-      <c r="J9" t="s" s="15">
+      <c r="J9" t="s" s="16">
         <v>72</v>
       </c>
-      <c r="K9" t="s" s="15">
+      <c r="K9" t="s" s="16">
         <v>64</v>
       </c>
-      <c r="L9" t="s" s="15">
+      <c r="L9" t="s" s="16">
         <v>73</v>
       </c>
-      <c r="M9" t="s" s="15">
+      <c r="M9" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N9" t="s" s="15">
+      <c r="N9" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P9" t="s" s="15">
+      <c r="P9" t="s" s="16">
         <v>74</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="s" s="15">
+      <c r="A10" t="s" s="16">
         <v>75</v>
       </c>
-      <c r="B10" t="s" s="15">
+      <c r="B10" t="s" s="16">
         <v>57</v>
       </c>
-      <c r="C10" t="s" s="15">
+      <c r="C10" t="s" s="16">
         <v>76</v>
       </c>
-      <c r="D10" t="s" s="15">
+      <c r="D10" t="s" s="16">
         <v>77</v>
       </c>
-      <c r="E10" t="s" s="15">
+      <c r="E10" t="s" s="16">
         <v>27</v>
       </c>
-      <c r="F10" t="s" s="15">
+      <c r="F10" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G10" t="s" s="15">
+      <c r="G10" t="s" s="16">
         <v>78</v>
       </c>
-      <c r="H10" t="s" s="15">
+      <c r="H10" t="s" s="16">
         <v>79</v>
       </c>
-      <c r="I10" t="s" s="15">
+      <c r="I10" t="s" s="16">
         <v>80</v>
       </c>
-      <c r="J10" t="s" s="15">
+      <c r="J10" t="s" s="16">
         <v>81</v>
       </c>
-      <c r="K10" t="s" s="15">
+      <c r="K10" t="s" s="16">
         <v>82</v>
       </c>
-      <c r="L10" t="s" s="15">
+      <c r="L10" t="s" s="16">
         <v>83</v>
       </c>
-      <c r="M10" t="s" s="15">
+      <c r="M10" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N10" t="s" s="15">
+      <c r="N10" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P10" t="s" s="15">
+      <c r="P10" t="s" s="16">
         <v>84</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="s" s="15">
+      <c r="A11" t="s" s="16">
         <v>85</v>
       </c>
-      <c r="B11" t="s" s="15">
+      <c r="B11" t="s" s="16">
         <v>57</v>
       </c>
-      <c r="C11" t="s" s="15">
+      <c r="C11" t="s" s="16">
         <v>76</v>
       </c>
-      <c r="D11" t="s" s="15">
+      <c r="D11" t="s" s="16">
         <v>86</v>
       </c>
-      <c r="E11" t="s" s="15">
+      <c r="E11" t="s" s="16">
         <v>27</v>
       </c>
-      <c r="F11" t="s" s="15">
+      <c r="F11" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G11" t="s" s="15">
+      <c r="G11" t="s" s="16">
         <v>69</v>
       </c>
-      <c r="H11" t="s" s="15">
+      <c r="H11" t="s" s="16">
         <v>87</v>
       </c>
-      <c r="I11" t="s" s="15">
+      <c r="I11" t="s" s="16">
         <v>88</v>
       </c>
-      <c r="J11" t="s" s="15">
+      <c r="J11" t="s" s="16">
         <v>89</v>
       </c>
-      <c r="K11" t="s" s="15">
+      <c r="K11" t="s" s="16">
         <v>82</v>
       </c>
-      <c r="L11" t="s" s="15">
+      <c r="L11" t="s" s="16">
         <v>90</v>
       </c>
-      <c r="M11" t="s" s="15">
+      <c r="M11" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N11" t="s" s="15">
+      <c r="N11" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P11" t="s" s="15">
+      <c r="P11" t="s" s="16">
         <v>91</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="s" s="15">
+      <c r="A12" t="s" s="16">
         <v>92</v>
       </c>
-      <c r="B12" t="s" s="15">
+      <c r="B12" t="s" s="16">
         <v>57</v>
       </c>
-      <c r="C12" t="s" s="15">
+      <c r="C12" t="s" s="16">
         <v>76</v>
       </c>
-      <c r="D12" t="s" s="15">
+      <c r="D12" t="s" s="16">
         <v>93</v>
       </c>
-      <c r="E12" t="s" s="15">
+      <c r="E12" t="s" s="16">
         <v>27</v>
       </c>
-      <c r="F12" t="s" s="15">
+      <c r="F12" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G12" t="s" s="15">
+      <c r="G12" t="s" s="16">
         <v>69</v>
       </c>
-      <c r="H12" t="s" s="15">
+      <c r="H12" t="s" s="16">
         <v>87</v>
       </c>
-      <c r="I12" t="s" s="15">
+      <c r="I12" t="s" s="16">
         <v>94</v>
       </c>
-      <c r="J12" t="s" s="15">
+      <c r="J12" t="s" s="16">
         <v>95</v>
       </c>
-      <c r="K12" t="s" s="15">
+      <c r="K12" t="s" s="16">
         <v>82</v>
       </c>
-      <c r="L12" t="s" s="15">
+      <c r="L12" t="s" s="16">
         <v>96</v>
       </c>
-      <c r="M12" t="s" s="15">
+      <c r="M12" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N12" t="s" s="15">
+      <c r="N12" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P12" t="s" s="15">
+      <c r="P12" t="s" s="16">
         <v>97</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="s" s="15">
+      <c r="A13" t="s" s="16">
         <v>98</v>
       </c>
-      <c r="B13" t="s" s="15">
+      <c r="B13" t="s" s="16">
         <v>57</v>
       </c>
-      <c r="C13" t="s" s="15">
+      <c r="C13" t="s" s="16">
         <v>99</v>
       </c>
-      <c r="D13" t="s" s="15">
+      <c r="D13" t="s" s="16">
         <v>100</v>
       </c>
-      <c r="E13" t="s" s="15">
+      <c r="E13" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F13" t="s" s="15">
+      <c r="F13" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G13" t="s" s="15">
+      <c r="G13" t="s" s="16">
         <v>69</v>
       </c>
-      <c r="H13" t="s" s="15">
+      <c r="H13" t="s" s="16">
         <v>101</v>
       </c>
-      <c r="I13" t="s" s="15">
+      <c r="I13" t="s" s="16">
         <v>102</v>
       </c>
-      <c r="J13" t="s" s="15">
+      <c r="J13" t="s" s="16">
         <v>103</v>
       </c>
-      <c r="K13" t="s" s="15">
+      <c r="K13" t="s" s="16">
         <v>64</v>
       </c>
-      <c r="L13" t="s" s="15">
+      <c r="L13" t="s" s="16">
         <v>104</v>
       </c>
-      <c r="M13" t="s" s="15">
+      <c r="M13" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N13" t="s" s="15">
+      <c r="N13" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P13" t="s" s="15">
+      <c r="P13" t="s" s="16">
         <v>105</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="s" s="15">
+      <c r="A14" t="s" s="16">
         <v>106</v>
       </c>
-      <c r="B14" t="s" s="15">
+      <c r="B14" t="s" s="16">
         <v>57</v>
       </c>
-      <c r="C14" t="s" s="15">
+      <c r="C14" t="s" s="16">
         <v>76</v>
       </c>
-      <c r="D14" t="s" s="15">
+      <c r="D14" t="s" s="16">
         <v>107</v>
       </c>
-      <c r="E14" t="s" s="15">
+      <c r="E14" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F14" t="s" s="15">
+      <c r="F14" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G14" t="s" s="15">
+      <c r="G14" t="s" s="16">
         <v>108</v>
       </c>
-      <c r="H14" t="s" s="15">
+      <c r="H14" t="s" s="16">
         <v>79</v>
       </c>
-      <c r="I14" t="s" s="15">
+      <c r="I14" t="s" s="16">
         <v>109</v>
       </c>
-      <c r="J14" t="s" s="15">
+      <c r="J14" t="s" s="16">
         <v>110</v>
       </c>
-      <c r="K14" t="s" s="15">
+      <c r="K14" t="s" s="16">
         <v>111</v>
       </c>
-      <c r="L14" t="s" s="15">
+      <c r="L14" t="s" s="16">
         <v>112</v>
       </c>
-      <c r="M14" t="s" s="15">
+      <c r="M14" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N14" t="s" s="15">
+      <c r="N14" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P14" t="s" s="15">
+      <c r="P14" t="s" s="16">
         <v>13</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="s" s="15">
+      <c r="A15" t="s" s="16">
         <v>113</v>
       </c>
-      <c r="B15" t="s" s="15">
+      <c r="B15" t="s" s="16">
         <v>57</v>
       </c>
-      <c r="C15" t="s" s="15">
+      <c r="C15" t="s" s="16">
         <v>76</v>
       </c>
-      <c r="D15" t="s" s="15">
+      <c r="D15" t="s" s="16">
         <v>114</v>
       </c>
-      <c r="E15" t="s" s="15">
+      <c r="E15" t="s" s="16">
         <v>27</v>
       </c>
-      <c r="F15" t="s" s="15">
+      <c r="F15" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G15" t="s" s="15">
+      <c r="G15" t="s" s="16">
         <v>108</v>
       </c>
-      <c r="H15" t="s" s="15">
+      <c r="H15" t="s" s="16">
         <v>79</v>
       </c>
-      <c r="I15" t="s" s="15">
+      <c r="I15" t="s" s="16">
         <v>115</v>
       </c>
-      <c r="J15" t="s" s="15">
+      <c r="J15" t="s" s="16">
         <v>116</v>
       </c>
-      <c r="K15" t="s" s="15">
+      <c r="K15" t="s" s="16">
         <v>117</v>
       </c>
-      <c r="L15" t="s" s="15">
+      <c r="L15" t="s" s="16">
         <v>118</v>
       </c>
-      <c r="M15" t="s" s="15">
+      <c r="M15" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N15" t="s" s="15">
+      <c r="N15" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P15" t="s" s="15">
+      <c r="P15" t="s" s="16">
         <v>119</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="s" s="15">
+      <c r="A16" t="s" s="16">
         <v>120</v>
       </c>
-      <c r="B16" t="s" s="15">
+      <c r="B16" t="s" s="16">
         <v>57</v>
       </c>
-      <c r="C16" t="s" s="15">
+      <c r="C16" t="s" s="16">
         <v>121</v>
       </c>
-      <c r="D16" t="s" s="15">
+      <c r="D16" t="s" s="16">
         <v>122</v>
       </c>
-      <c r="E16" t="s" s="15">
+      <c r="E16" t="s" s="16">
         <v>27</v>
       </c>
-      <c r="F16" t="s" s="15">
+      <c r="F16" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G16" t="s" s="15">
+      <c r="G16" t="s" s="16">
         <v>108</v>
       </c>
-      <c r="H16" t="s" s="15">
+      <c r="H16" t="s" s="16">
         <v>123</v>
       </c>
-      <c r="I16" t="s" s="15">
+      <c r="I16" t="s" s="16">
         <v>124</v>
       </c>
-      <c r="J16" t="s" s="15">
+      <c r="J16" t="s" s="16">
         <v>125</v>
       </c>
-      <c r="K16" t="s" s="15">
+      <c r="K16" t="s" s="16">
         <v>117</v>
       </c>
-      <c r="L16" t="s" s="15">
+      <c r="L16" t="s" s="16">
         <v>126</v>
       </c>
-      <c r="M16" t="s" s="15">
+      <c r="M16" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N16" t="s" s="15">
+      <c r="N16" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P16" t="s" s="15">
+      <c r="P16" t="s" s="16">
         <v>127</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="s" s="15">
+      <c r="A17" t="s" s="16">
         <v>128</v>
       </c>
-      <c r="B17" t="s" s="15">
+      <c r="B17" t="s" s="16">
         <v>129</v>
       </c>
-      <c r="C17" t="s" s="15">
+      <c r="C17" t="s" s="16">
         <v>130</v>
       </c>
-      <c r="D17" t="s" s="15">
+      <c r="D17" t="s" s="16">
         <v>131</v>
       </c>
-      <c r="E17" t="s" s="15">
+      <c r="E17" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F17" t="s" s="15">
+      <c r="F17" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G17" t="s" s="15">
+      <c r="G17" t="s" s="16">
         <v>18</v>
       </c>
-      <c r="H17" t="s" s="15">
+      <c r="H17" t="s" s="16">
         <v>132</v>
       </c>
-      <c r="I17" t="s" s="15">
+      <c r="I17" t="s" s="16">
         <v>133</v>
       </c>
-      <c r="J17" t="s" s="15">
+      <c r="J17" t="s" s="16">
         <v>134</v>
       </c>
-      <c r="K17" t="s" s="15">
+      <c r="K17" t="s" s="16">
         <v>135</v>
       </c>
-      <c r="L17" t="s" s="15">
+      <c r="L17" t="s" s="16">
         <v>136</v>
       </c>
-      <c r="M17" t="s" s="15">
+      <c r="M17" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N17" t="s" s="15">
+      <c r="N17" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P17" t="s" s="15">
+      <c r="P17" t="s" s="16">
         <v>137</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="s" s="15">
+      <c r="A18" t="s" s="16">
         <v>138</v>
       </c>
-      <c r="B18" t="s" s="15">
+      <c r="B18" t="s" s="16">
         <v>129</v>
       </c>
-      <c r="C18" t="s" s="15">
+      <c r="C18" t="s" s="16">
         <v>139</v>
       </c>
-      <c r="D18" t="s" s="15">
+      <c r="D18" t="s" s="16">
         <v>140</v>
       </c>
-      <c r="E18" t="s" s="15">
+      <c r="E18" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F18" t="s" s="15">
+      <c r="F18" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G18" t="s" s="15">
+      <c r="G18" t="s" s="16">
         <v>18</v>
       </c>
-      <c r="H18" t="s" s="15">
+      <c r="H18" t="s" s="16">
         <v>141</v>
       </c>
-      <c r="I18" t="s" s="15">
+      <c r="I18" t="s" s="16">
         <v>142</v>
       </c>
-      <c r="J18" t="s" s="15">
+      <c r="J18" t="s" s="16">
         <v>143</v>
       </c>
-      <c r="K18" t="s" s="15">
+      <c r="K18" t="s" s="16">
         <v>144</v>
       </c>
-      <c r="L18" t="s" s="15">
+      <c r="L18" t="s" s="16">
         <v>145</v>
       </c>
-      <c r="M18" t="s" s="15">
+      <c r="M18" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N18" t="s" s="15">
+      <c r="N18" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P18" t="s" s="15">
+      <c r="P18" t="s" s="16">
         <v>13</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="s" s="15">
+      <c r="A19" t="s" s="16">
         <v>146</v>
       </c>
-      <c r="B19" t="s" s="15">
+      <c r="B19" t="s" s="16">
         <v>129</v>
       </c>
-      <c r="C19" t="s" s="15">
+      <c r="C19" t="s" s="16">
         <v>139</v>
       </c>
-      <c r="D19" t="s" s="15">
+      <c r="D19" t="s" s="16">
         <v>147</v>
       </c>
-      <c r="E19" t="s" s="15">
+      <c r="E19" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F19" t="s" s="15">
+      <c r="F19" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G19" t="s" s="15">
+      <c r="G19" t="s" s="16">
         <v>148</v>
       </c>
-      <c r="H19" t="s" s="15">
+      <c r="H19" t="s" s="16">
         <v>149</v>
       </c>
-      <c r="I19" t="s" s="15">
+      <c r="I19" t="s" s="16">
         <v>150</v>
       </c>
-      <c r="J19" t="s" s="15">
+      <c r="J19" t="s" s="16">
         <v>151</v>
       </c>
-      <c r="K19" t="s" s="15">
+      <c r="K19" t="s" s="16">
         <v>111</v>
       </c>
-      <c r="L19" t="s" s="15">
+      <c r="L19" t="s" s="16">
         <v>152</v>
       </c>
-      <c r="M19" t="s" s="15">
+      <c r="M19" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N19" t="s" s="15">
+      <c r="N19" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P19" t="s" s="15">
+      <c r="P19" t="s" s="16">
         <v>153</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="s" s="15">
+      <c r="A20" t="s" s="16">
         <v>154</v>
       </c>
-      <c r="B20" t="s" s="15">
+      <c r="B20" t="s" s="16">
         <v>129</v>
       </c>
-      <c r="C20" t="s" s="15">
+      <c r="C20" t="s" s="16">
         <v>139</v>
       </c>
-      <c r="D20" t="s" s="15">
+      <c r="D20" t="s" s="16">
         <v>155</v>
       </c>
-      <c r="E20" t="s" s="15">
+      <c r="E20" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F20" t="s" s="15">
+      <c r="F20" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G20" t="s" s="15">
+      <c r="G20" t="s" s="16">
         <v>148</v>
       </c>
-      <c r="H20" t="s" s="15">
+      <c r="H20" t="s" s="16">
         <v>156</v>
       </c>
-      <c r="I20" t="s" s="15">
+      <c r="I20" t="s" s="16">
         <v>157</v>
       </c>
-      <c r="J20" t="s" s="15">
+      <c r="J20" t="s" s="16">
         <v>158</v>
       </c>
-      <c r="K20" t="s" s="15">
+      <c r="K20" t="s" s="16">
         <v>111</v>
       </c>
-      <c r="L20" t="s" s="15">
+      <c r="L20" t="s" s="16">
         <v>159</v>
       </c>
-      <c r="M20" t="s" s="15">
+      <c r="M20" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N20" t="s" s="15">
+      <c r="N20" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P20" t="s" s="15">
+      <c r="P20" t="s" s="16">
         <v>160</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="s" s="15">
+      <c r="A21" t="s" s="16">
         <v>161</v>
       </c>
-      <c r="B21" t="s" s="15">
+      <c r="B21" t="s" s="16">
         <v>129</v>
       </c>
-      <c r="C21" t="s" s="15">
+      <c r="C21" t="s" s="16">
         <v>139</v>
       </c>
-      <c r="D21" t="s" s="15">
+      <c r="D21" t="s" s="16">
         <v>162</v>
       </c>
-      <c r="E21" t="s" s="15">
+      <c r="E21" t="s" s="16">
         <v>27</v>
       </c>
-      <c r="F21" t="s" s="15">
+      <c r="F21" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G21" t="s" s="15">
+      <c r="G21" t="s" s="16">
         <v>18</v>
       </c>
-      <c r="H21" t="s" s="15">
+      <c r="H21" t="s" s="16">
         <v>163</v>
       </c>
-      <c r="I21" t="s" s="15">
+      <c r="I21" t="s" s="16">
         <v>164</v>
       </c>
-      <c r="J21" t="s" s="15">
+      <c r="J21" t="s" s="16">
         <v>165</v>
       </c>
-      <c r="K21" t="s" s="15">
+      <c r="K21" t="s" s="16">
         <v>166</v>
       </c>
-      <c r="L21" t="s" s="15">
+      <c r="L21" t="s" s="16">
         <v>167</v>
       </c>
-      <c r="M21" t="s" s="15">
+      <c r="M21" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N21" t="s" s="15">
+      <c r="N21" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P21" t="s" s="15">
+      <c r="P21" t="s" s="16">
         <v>168</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="s" s="15">
+      <c r="A22" t="s" s="16">
         <v>169</v>
       </c>
-      <c r="B22" t="s" s="15">
+      <c r="B22" t="s" s="16">
         <v>129</v>
       </c>
-      <c r="C22" t="s" s="15">
+      <c r="C22" t="s" s="16">
         <v>170</v>
       </c>
-      <c r="D22" t="s" s="15">
+      <c r="D22" t="s" s="16">
         <v>171</v>
       </c>
-      <c r="E22" t="s" s="15">
+      <c r="E22" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F22" t="s" s="15">
+      <c r="F22" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G22" t="s" s="15">
+      <c r="G22" t="s" s="16">
         <v>18</v>
       </c>
-      <c r="H22" t="s" s="15">
+      <c r="H22" t="s" s="16">
         <v>172</v>
       </c>
-      <c r="I22" t="s" s="15">
+      <c r="I22" t="s" s="16">
         <v>173</v>
       </c>
-      <c r="J22" t="s" s="15">
+      <c r="J22" t="s" s="16">
         <v>174</v>
       </c>
-      <c r="K22" t="s" s="15">
+      <c r="K22" t="s" s="16">
         <v>144</v>
       </c>
-      <c r="L22" t="s" s="15">
+      <c r="L22" t="s" s="16">
         <v>175</v>
       </c>
-      <c r="M22" t="s" s="15">
+      <c r="M22" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N22" t="s" s="15">
+      <c r="N22" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P22" t="s" s="15">
+      <c r="P22" t="s" s="16">
         <v>176</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="s" s="15">
+      <c r="A23" t="s" s="16">
         <v>177</v>
       </c>
-      <c r="B23" t="s" s="15">
+      <c r="B23" t="s" s="16">
         <v>129</v>
       </c>
-      <c r="C23" t="s" s="15">
+      <c r="C23" t="s" s="16">
         <v>170</v>
       </c>
-      <c r="D23" t="s" s="15">
+      <c r="D23" t="s" s="16">
         <v>178</v>
       </c>
-      <c r="E23" t="s" s="15">
+      <c r="E23" t="s" s="16">
         <v>27</v>
       </c>
-      <c r="F23" t="s" s="15">
+      <c r="F23" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G23" t="s" s="15">
+      <c r="G23" t="s" s="16">
         <v>179</v>
       </c>
-      <c r="H23" t="s" s="15">
+      <c r="H23" t="s" s="16">
         <v>180</v>
       </c>
-      <c r="I23" t="s" s="15">
+      <c r="I23" t="s" s="16">
         <v>181</v>
       </c>
-      <c r="J23" t="s" s="15">
+      <c r="J23" t="s" s="16">
         <v>182</v>
       </c>
-      <c r="K23" t="s" s="15">
+      <c r="K23" t="s" s="16">
         <v>183</v>
       </c>
-      <c r="L23" t="s" s="15">
+      <c r="L23" t="s" s="16">
         <v>184</v>
       </c>
-      <c r="M23" t="s" s="15">
+      <c r="M23" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N23" t="s" s="15">
+      <c r="N23" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P23" t="s" s="15">
+      <c r="P23" t="s" s="16">
         <v>185</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="s" s="15">
+      <c r="A24" t="s" s="16">
         <v>186</v>
       </c>
-      <c r="B24" t="s" s="15">
+      <c r="B24" t="s" s="16">
         <v>129</v>
       </c>
-      <c r="C24" t="s" s="15">
+      <c r="C24" t="s" s="16">
         <v>170</v>
       </c>
-      <c r="D24" t="s" s="15">
+      <c r="D24" t="s" s="16">
         <v>187</v>
       </c>
-      <c r="E24" t="s" s="15">
+      <c r="E24" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F24" t="s" s="15">
+      <c r="F24" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G24" t="s" s="15">
+      <c r="G24" t="s" s="16">
         <v>179</v>
       </c>
-      <c r="H24" t="s" s="15">
+      <c r="H24" t="s" s="16">
         <v>188</v>
       </c>
-      <c r="I24" t="s" s="15">
+      <c r="I24" t="s" s="16">
         <v>189</v>
       </c>
-      <c r="J24" t="s" s="15">
+      <c r="J24" t="s" s="16">
         <v>190</v>
       </c>
-      <c r="K24" t="s" s="15">
+      <c r="K24" t="s" s="16">
         <v>135</v>
       </c>
-      <c r="L24" t="s" s="15">
+      <c r="L24" t="s" s="16">
         <v>191</v>
       </c>
-      <c r="M24" t="s" s="15">
+      <c r="M24" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N24" t="s" s="15">
+      <c r="N24" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P24" t="s" s="15">
+      <c r="P24" t="s" s="16">
         <v>13</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="s" s="15">
+      <c r="A25" t="s" s="16">
         <v>192</v>
       </c>
-      <c r="B25" t="s" s="15">
+      <c r="B25" t="s" s="16">
         <v>129</v>
       </c>
-      <c r="C25" t="s" s="15">
+      <c r="C25" t="s" s="16">
         <v>170</v>
       </c>
-      <c r="D25" t="s" s="15">
+      <c r="D25" t="s" s="16">
         <v>193</v>
       </c>
-      <c r="E25" t="s" s="15">
+      <c r="E25" t="s" s="16">
         <v>27</v>
       </c>
-      <c r="F25" t="s" s="15">
+      <c r="F25" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G25" t="s" s="15">
+      <c r="G25" t="s" s="16">
         <v>179</v>
       </c>
-      <c r="H25" t="s" s="15">
+      <c r="H25" t="s" s="16">
         <v>194</v>
       </c>
-      <c r="I25" t="s" s="15">
+      <c r="I25" t="s" s="16">
         <v>195</v>
       </c>
-      <c r="J25" t="s" s="15">
+      <c r="J25" t="s" s="16">
         <v>196</v>
       </c>
-      <c r="K25" t="s" s="15">
+      <c r="K25" t="s" s="16">
         <v>166</v>
       </c>
-      <c r="L25" t="s" s="15">
+      <c r="L25" t="s" s="16">
         <v>197</v>
       </c>
-      <c r="M25" t="s" s="15">
+      <c r="M25" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N25" t="s" s="15">
+      <c r="N25" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P25" t="s" s="15">
+      <c r="P25" t="s" s="16">
         <v>13</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="s" s="15">
+      <c r="A26" t="s" s="16">
         <v>198</v>
       </c>
-      <c r="B26" t="s" s="15">
+      <c r="B26" t="s" s="16">
         <v>129</v>
       </c>
-      <c r="C26" t="s" s="15">
+      <c r="C26" t="s" s="16">
         <v>170</v>
       </c>
-      <c r="D26" t="s" s="15">
+      <c r="D26" t="s" s="16">
         <v>199</v>
       </c>
-      <c r="E26" t="s" s="15">
+      <c r="E26" t="s" s="16">
         <v>27</v>
       </c>
-      <c r="F26" t="s" s="15">
+      <c r="F26" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G26" t="s" s="15">
+      <c r="G26" t="s" s="16">
         <v>179</v>
       </c>
-      <c r="H26" t="s" s="15">
+      <c r="H26" t="s" s="16">
         <v>200</v>
       </c>
-      <c r="I26" t="s" s="15">
+      <c r="I26" t="s" s="16">
         <v>201</v>
       </c>
-      <c r="J26" t="s" s="15">
+      <c r="J26" t="s" s="16">
         <v>202</v>
       </c>
-      <c r="K26" t="s" s="15">
+      <c r="K26" t="s" s="16">
         <v>166</v>
       </c>
-      <c r="L26" t="s" s="15">
+      <c r="L26" t="s" s="16">
         <v>203</v>
       </c>
-      <c r="M26" t="s" s="15">
+      <c r="M26" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N26" t="s" s="15">
+      <c r="N26" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P26" t="s" s="15">
+      <c r="P26" t="s" s="16">
         <v>204</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="s" s="15">
+      <c r="A27" t="s" s="16">
         <v>205</v>
       </c>
-      <c r="B27" t="s" s="15">
+      <c r="B27" t="s" s="16">
         <v>129</v>
       </c>
-      <c r="C27" t="s" s="15">
+      <c r="C27" t="s" s="16">
         <v>170</v>
       </c>
-      <c r="D27" t="s" s="15">
+      <c r="D27" t="s" s="16">
         <v>206</v>
       </c>
-      <c r="E27" t="s" s="15">
+      <c r="E27" t="s" s="16">
         <v>27</v>
       </c>
-      <c r="F27" t="s" s="15">
+      <c r="F27" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G27" t="s" s="15">
+      <c r="G27" t="s" s="16">
         <v>179</v>
       </c>
-      <c r="H27" t="s" s="15">
+      <c r="H27" t="s" s="16">
         <v>207</v>
       </c>
-      <c r="I27" t="s" s="15">
+      <c r="I27" t="s" s="16">
         <v>208</v>
       </c>
-      <c r="J27" t="s" s="15">
+      <c r="J27" t="s" s="16">
         <v>209</v>
       </c>
-      <c r="K27" t="s" s="15">
+      <c r="K27" t="s" s="16">
         <v>166</v>
       </c>
-      <c r="L27" t="s" s="15">
+      <c r="L27" t="s" s="16">
         <v>210</v>
       </c>
-      <c r="M27" t="s" s="15">
+      <c r="M27" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N27" t="s" s="15">
+      <c r="N27" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P27" t="s" s="15">
+      <c r="P27" t="s" s="16">
         <v>211</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="s" s="15">
+      <c r="A28" t="s" s="16">
         <v>212</v>
       </c>
-      <c r="B28" t="s" s="15">
+      <c r="B28" t="s" s="16">
         <v>213</v>
       </c>
-      <c r="C28" t="s" s="15">
+      <c r="C28" t="s" s="16">
         <v>214</v>
       </c>
-      <c r="D28" t="s" s="15">
+      <c r="D28" t="s" s="16">
         <v>215</v>
       </c>
-      <c r="E28" t="s" s="15">
+      <c r="E28" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F28" t="s" s="15">
+      <c r="F28" t="s" s="16">
         <v>216</v>
       </c>
-      <c r="G28" t="s" s="15">
+      <c r="G28" t="s" s="16">
         <v>217</v>
       </c>
-      <c r="H28" t="s" s="15">
+      <c r="H28" t="s" s="16">
         <v>218</v>
       </c>
-      <c r="I28" t="s" s="15">
+      <c r="I28" t="s" s="16">
         <v>219</v>
       </c>
-      <c r="J28" t="s" s="15">
+      <c r="J28" t="s" s="16">
         <v>220</v>
       </c>
-      <c r="K28" t="s" s="15">
+      <c r="K28" t="s" s="16">
         <v>221</v>
       </c>
-      <c r="L28" t="s" s="15">
+      <c r="L28" t="s" s="16">
         <v>222</v>
       </c>
-      <c r="M28" t="s" s="15">
+      <c r="M28" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N28" t="s" s="15">
+      <c r="N28" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P28" t="s" s="15">
+      <c r="P28" t="s" s="16">
         <v>223</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="s" s="15">
+      <c r="A29" t="s" s="16">
         <v>224</v>
       </c>
-      <c r="B29" t="s" s="15">
+      <c r="B29" t="s" s="16">
         <v>213</v>
       </c>
-      <c r="C29" t="s" s="15">
+      <c r="C29" t="s" s="16">
         <v>214</v>
       </c>
-      <c r="D29" t="s" s="15">
+      <c r="D29" t="s" s="16">
         <v>225</v>
       </c>
-      <c r="E29" t="s" s="15">
+      <c r="E29" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F29" t="s" s="15">
+      <c r="F29" t="s" s="16">
         <v>216</v>
       </c>
-      <c r="G29" t="s" s="15">
+      <c r="G29" t="s" s="16">
         <v>226</v>
       </c>
-      <c r="H29" t="s" s="15">
+      <c r="H29" t="s" s="16">
         <v>227</v>
       </c>
-      <c r="I29" t="s" s="15">
+      <c r="I29" t="s" s="16">
         <v>228</v>
       </c>
-      <c r="J29" t="s" s="15">
+      <c r="J29" t="s" s="16">
         <v>229</v>
       </c>
-      <c r="K29" t="s" s="15">
+      <c r="K29" t="s" s="16">
         <v>230</v>
       </c>
-      <c r="L29" t="s" s="15">
+      <c r="L29" t="s" s="16">
         <v>231</v>
       </c>
-      <c r="M29" t="s" s="15">
+      <c r="M29" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N29" t="s" s="15">
+      <c r="N29" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P29" t="s" s="15">
+      <c r="P29" t="s" s="16">
         <v>232</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="s" s="15">
+      <c r="A30" t="s" s="16">
         <v>233</v>
       </c>
-      <c r="B30" t="s" s="15">
+      <c r="B30" t="s" s="16">
         <v>213</v>
       </c>
-      <c r="C30" t="s" s="15">
+      <c r="C30" t="s" s="16">
         <v>214</v>
       </c>
-      <c r="D30" t="s" s="15">
+      <c r="D30" t="s" s="16">
         <v>234</v>
       </c>
-      <c r="E30" t="s" s="15">
+      <c r="E30" t="s" s="16">
         <v>27</v>
       </c>
-      <c r="F30" t="s" s="15">
+      <c r="F30" t="s" s="16">
         <v>216</v>
       </c>
-      <c r="G30" t="s" s="15">
+      <c r="G30" t="s" s="16">
         <v>235</v>
       </c>
-      <c r="H30" t="s" s="15">
+      <c r="H30" t="s" s="16">
         <v>236</v>
       </c>
-      <c r="I30" t="s" s="15">
+      <c r="I30" t="s" s="16">
         <v>237</v>
       </c>
-      <c r="J30" t="s" s="15">
+      <c r="J30" t="s" s="16">
         <v>238</v>
       </c>
-      <c r="K30" t="s" s="15">
+      <c r="K30" t="s" s="16">
         <v>239</v>
       </c>
-      <c r="L30" t="s" s="15">
+      <c r="L30" t="s" s="16">
         <v>240</v>
       </c>
-      <c r="M30" t="s" s="15">
+      <c r="M30" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N30" t="s" s="15">
+      <c r="N30" t="s" s="16">
         <v>344</v>
       </c>
-      <c r="P30" t="s" s="15">
+      <c r="P30" t="s" s="16">
         <v>242</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="s" s="15">
+      <c r="A31" t="s" s="16">
         <v>243</v>
       </c>
-      <c r="B31" t="s" s="15">
+      <c r="B31" t="s" s="16">
         <v>213</v>
       </c>
-      <c r="C31" t="s" s="15">
+      <c r="C31" t="s" s="16">
         <v>244</v>
       </c>
-      <c r="D31" t="s" s="15">
+      <c r="D31" t="s" s="16">
         <v>245</v>
       </c>
-      <c r="E31" t="s" s="15">
+      <c r="E31" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F31" t="s" s="15">
+      <c r="F31" t="s" s="16">
         <v>216</v>
       </c>
-      <c r="G31" t="s" s="15">
+      <c r="G31" t="s" s="16">
         <v>18</v>
       </c>
-      <c r="H31" t="s" s="15">
+      <c r="H31" t="s" s="16">
         <v>246</v>
       </c>
-      <c r="I31" t="s" s="15">
+      <c r="I31" t="s" s="16">
         <v>247</v>
       </c>
-      <c r="J31" t="s" s="15">
+      <c r="J31" t="s" s="16">
         <v>248</v>
       </c>
-      <c r="K31" t="s" s="15">
+      <c r="K31" t="s" s="16">
         <v>221</v>
       </c>
-      <c r="L31" t="s" s="15">
+      <c r="L31" t="s" s="16">
         <v>249</v>
       </c>
-      <c r="M31" t="s" s="15">
+      <c r="M31" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N31" t="s" s="15">
+      <c r="N31" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P31" t="s" s="15">
+      <c r="P31" t="s" s="16">
         <v>250</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="s" s="15">
+      <c r="A32" t="s" s="16">
         <v>251</v>
       </c>
-      <c r="B32" t="s" s="15">
+      <c r="B32" t="s" s="16">
         <v>213</v>
       </c>
-      <c r="C32" t="s" s="15">
+      <c r="C32" t="s" s="16">
         <v>244</v>
       </c>
-      <c r="D32" t="s" s="15">
+      <c r="D32" t="s" s="16">
         <v>252</v>
       </c>
-      <c r="E32" t="s" s="15">
+      <c r="E32" t="s" s="16">
         <v>27</v>
       </c>
-      <c r="F32" t="s" s="15">
+      <c r="F32" t="s" s="16">
         <v>216</v>
       </c>
-      <c r="G32" t="s" s="15">
+      <c r="G32" t="s" s="16">
         <v>18</v>
       </c>
-      <c r="H32" t="s" s="15">
+      <c r="H32" t="s" s="16">
         <v>253</v>
       </c>
-      <c r="I32" t="s" s="15">
+      <c r="I32" t="s" s="16">
         <v>254</v>
       </c>
-      <c r="J32" t="s" s="15">
+      <c r="J32" t="s" s="16">
         <v>255</v>
       </c>
-      <c r="K32" t="s" s="15">
+      <c r="K32" t="s" s="16">
         <v>230</v>
       </c>
-      <c r="L32" t="s" s="15">
+      <c r="L32" t="s" s="16">
         <v>256</v>
       </c>
-      <c r="M32" t="s" s="15">
+      <c r="M32" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N32" t="s" s="15">
+      <c r="N32" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P32" t="s" s="15">
+      <c r="P32" t="s" s="16">
         <v>13</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="s" s="15">
+      <c r="A33" t="s" s="16">
         <v>257</v>
       </c>
-      <c r="B33" t="s" s="15">
+      <c r="B33" t="s" s="16">
         <v>213</v>
       </c>
-      <c r="C33" t="s" s="15">
+      <c r="C33" t="s" s="16">
         <v>214</v>
       </c>
-      <c r="D33" t="s" s="15">
-        <v>258</v>
-      </c>
-      <c r="E33" t="s" s="15">
+      <c r="D33" t="s" s="16">
+        <v>350</v>
+      </c>
+      <c r="E33" t="s" s="16">
         <v>27</v>
       </c>
-      <c r="F33" t="s" s="15">
+      <c r="F33" t="s" s="16">
         <v>216</v>
       </c>
-      <c r="G33" t="s" s="15">
+      <c r="G33" t="s" s="16">
         <v>259</v>
       </c>
-      <c r="H33" t="s" s="15">
-        <v>260</v>
-      </c>
-      <c r="I33" t="s" s="15">
-        <v>261</v>
-      </c>
-      <c r="J33" t="s" s="15">
-        <v>262</v>
-      </c>
-      <c r="K33" t="s" s="15">
+      <c r="H33" t="s" s="16">
+        <v>351</v>
+      </c>
+      <c r="I33" t="s" s="16">
+        <v>352</v>
+      </c>
+      <c r="J33" t="s" s="16">
+        <v>353</v>
+      </c>
+      <c r="K33" t="s" s="16">
         <v>230</v>
       </c>
-      <c r="L33" t="s" s="15">
-        <v>263</v>
-      </c>
-      <c r="M33" t="s" s="15">
+      <c r="L33" t="s" s="16">
+        <v>354</v>
+      </c>
+      <c r="M33" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N33" t="s" s="15">
+      <c r="N33" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P33" t="s" s="15">
-        <v>264</v>
+      <c r="P33" t="s" s="16">
+        <v>355</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="s" s="15">
+      <c r="A34" t="s" s="16">
         <v>265</v>
       </c>
-      <c r="B34" t="s" s="15">
+      <c r="B34" t="s" s="16">
         <v>266</v>
       </c>
-      <c r="C34" t="s" s="15">
+      <c r="C34" t="s" s="16">
         <v>121</v>
       </c>
-      <c r="D34" t="s" s="15">
+      <c r="D34" t="s" s="16">
         <v>267</v>
       </c>
-      <c r="E34" t="s" s="15">
+      <c r="E34" t="s" s="16">
         <v>4</v>
       </c>
-      <c r="F34" t="s" s="15">
+      <c r="F34" t="s" s="16">
         <v>5</v>
       </c>
-      <c r="G34" t="s" s="15">
+      <c r="G34" t="s" s="16">
         <v>268</v>
       </c>
-      <c r="H34" t="s" s="15">
+      <c r="H34" t="s" s="16">
         <v>269</v>
       </c>
-      <c r="I34" t="s" s="15">
+      <c r="I34" t="s" s="16">
         <v>270</v>
       </c>
-      <c r="J34" t="s" s="15">
+      <c r="J34" t="s" s="16">
         <v>271</v>
       </c>
-      <c r="K34" t="s" s="15">
+      <c r="K34" t="s" s="16">
         <v>272</v>
       </c>
-      <c r="L34" t="s" s="15">
+      <c r="L34" t="s" s="16">
         <v>273</v>
       </c>
-      <c r="M34" t="s" s="15">
+      <c r="M34" t="s" s="16">
         <v>12</v>
       </c>
-      <c r="N34" t="s" s="15">
+      <c r="N34" t="s" s="16">
         <v>343</v>
       </c>
-      <c r="P34" t="s" s="15">
+      <c r="P34" t="s" s="16">
         <v>274</v>
       </c>
     </row>
@@ -3718,240 +3752,240 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="15">
+      <c r="A2" t="s" s="16">
         <v>275</v>
       </c>
-      <c r="B2" t="s" s="15">
+      <c r="B2" t="s" s="16">
         <v>2</v>
       </c>
-      <c r="C2" t="s" s="15">
+      <c r="C2" t="s" s="16">
         <v>0</v>
       </c>
-      <c r="D2" t="s" s="15">
+      <c r="D2" t="s" s="16">
         <v>276</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="15">
+      <c r="A3" t="s" s="16">
         <v>275</v>
       </c>
-      <c r="B3" t="s" s="15">
+      <c r="B3" t="s" s="16">
         <v>16</v>
       </c>
-      <c r="C3" t="s" s="15">
+      <c r="C3" t="s" s="16">
         <v>277</v>
       </c>
-      <c r="D3" t="s" s="15">
+      <c r="D3" t="s" s="16">
         <v>278</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s" s="15">
+      <c r="A4" t="s" s="16">
         <v>275</v>
       </c>
-      <c r="B4" t="s" s="15">
+      <c r="B4" t="s" s="16">
         <v>42</v>
       </c>
-      <c r="C4" t="s" s="15">
+      <c r="C4" t="s" s="16">
         <v>41</v>
       </c>
-      <c r="D4" t="s" s="15">
+      <c r="D4" t="s" s="16">
         <v>276</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s" s="15">
+      <c r="A5" t="s" s="16">
         <v>279</v>
       </c>
-      <c r="B5" t="s" s="15">
+      <c r="B5" t="s" s="16">
         <v>58</v>
       </c>
-      <c r="C5" t="s" s="15">
+      <c r="C5" t="s" s="16">
         <v>280</v>
       </c>
-      <c r="D5" t="s" s="15">
+      <c r="D5" t="s" s="16">
         <v>281</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s" s="15">
+      <c r="A6" t="s" s="16">
         <v>279</v>
       </c>
-      <c r="B6" t="s" s="15">
+      <c r="B6" t="s" s="16">
         <v>76</v>
       </c>
-      <c r="C6" t="s" s="15">
+      <c r="C6" t="s" s="16">
         <v>282</v>
       </c>
-      <c r="D6" t="s" s="15">
+      <c r="D6" t="s" s="16">
         <v>283</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s" s="15">
+      <c r="A7" t="s" s="16">
         <v>279</v>
       </c>
-      <c r="B7" t="s" s="15">
+      <c r="B7" t="s" s="16">
         <v>99</v>
       </c>
-      <c r="C7" t="s" s="15">
+      <c r="C7" t="s" s="16">
         <v>98</v>
       </c>
-      <c r="D7" t="s" s="15">
+      <c r="D7" t="s" s="16">
         <v>276</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="s" s="15">
+      <c r="A8" t="s" s="16">
         <v>284</v>
       </c>
-      <c r="B8" t="s" s="15">
+      <c r="B8" t="s" s="16">
         <v>130</v>
       </c>
-      <c r="C8" t="s" s="15">
+      <c r="C8" t="s" s="16">
         <v>285</v>
       </c>
-      <c r="D8" t="s" s="15">
+      <c r="D8" t="s" s="16">
         <v>276</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="s" s="15">
+      <c r="A9" t="s" s="16">
         <v>284</v>
       </c>
-      <c r="B9" t="s" s="15">
+      <c r="B9" t="s" s="16">
         <v>139</v>
       </c>
-      <c r="C9" t="s" s="15">
+      <c r="C9" t="s" s="16">
         <v>286</v>
       </c>
-      <c r="D9" t="s" s="15">
+      <c r="D9" t="s" s="16">
         <v>278</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="s" s="15">
+      <c r="A10" t="s" s="16">
         <v>284</v>
       </c>
-      <c r="B10" t="s" s="15">
+      <c r="B10" t="s" s="16">
         <v>170</v>
       </c>
-      <c r="C10" t="s" s="15">
+      <c r="C10" t="s" s="16">
         <v>287</v>
       </c>
-      <c r="D10" t="s" s="15">
+      <c r="D10" t="s" s="16">
         <v>288</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="s" s="15">
+      <c r="A11" t="s" s="16">
         <v>289</v>
       </c>
-      <c r="B11" t="s" s="15">
+      <c r="B11" t="s" s="16">
         <v>290</v>
       </c>
-      <c r="C11" t="s" s="15">
+      <c r="C11" t="s" s="16">
         <v>291</v>
       </c>
-      <c r="D11" t="s" s="15">
+      <c r="D11" t="s" s="16">
         <v>278</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="s" s="15">
+      <c r="A12" t="s" s="16">
         <v>289</v>
       </c>
-      <c r="B12" t="s" s="15">
+      <c r="B12" t="s" s="16">
         <v>292</v>
       </c>
-      <c r="C12" t="s" s="15">
+      <c r="C12" t="s" s="16">
         <v>293</v>
       </c>
-      <c r="D12" t="s" s="15">
+      <c r="D12" t="s" s="16">
         <v>281</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="s" s="15">
+      <c r="A13" t="s" s="16">
         <v>289</v>
       </c>
-      <c r="B13" t="s" s="15">
+      <c r="B13" t="s" s="16">
         <v>294</v>
       </c>
-      <c r="C13" t="s" s="15">
+      <c r="C13" t="s" s="16">
         <v>295</v>
       </c>
-      <c r="D13" t="s" s="15">
+      <c r="D13" t="s" s="16">
         <v>296</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="s" s="15">
+      <c r="A14" t="s" s="16">
         <v>289</v>
       </c>
-      <c r="B14" t="s" s="15">
+      <c r="B14" t="s" s="16">
         <v>297</v>
       </c>
-      <c r="C14" t="s" s="15">
+      <c r="C14" t="s" s="16">
         <v>298</v>
       </c>
-      <c r="D14" t="s" s="15">
+      <c r="D14" t="s" s="16">
         <v>296</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="s" s="15">
+      <c r="A15" t="s" s="16">
         <v>299</v>
       </c>
-      <c r="B15" t="s" s="15">
+      <c r="B15" t="s" s="16">
         <v>300</v>
       </c>
-      <c r="C15" t="s" s="15">
+      <c r="C15" t="s" s="16">
         <v>301</v>
       </c>
-      <c r="D15" t="s" s="15">
+      <c r="D15" t="s" s="16">
         <v>288</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="s" s="15">
+      <c r="A16" t="s" s="16">
         <v>299</v>
       </c>
-      <c r="B16" t="s" s="15">
+      <c r="B16" t="s" s="16">
         <v>302</v>
       </c>
-      <c r="C16" t="s" s="15">
+      <c r="C16" t="s" s="16">
         <v>303</v>
       </c>
-      <c r="D16" t="s" s="15">
+      <c r="D16" t="s" s="16">
         <v>288</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="s" s="15">
+      <c r="A17" t="s" s="16">
         <v>299</v>
       </c>
-      <c r="B17" t="s" s="15">
+      <c r="B17" t="s" s="16">
         <v>304</v>
       </c>
-      <c r="C17" t="s" s="15">
+      <c r="C17" t="s" s="16">
         <v>305</v>
       </c>
-      <c r="D17" t="s" s="15">
+      <c r="D17" t="s" s="16">
         <v>276</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="s" s="15">
+      <c r="A18" t="s" s="16">
         <v>299</v>
       </c>
-      <c r="B18" t="s" s="15">
+      <c r="B18" t="s" s="16">
         <v>306</v>
       </c>
-      <c r="C18" t="s" s="15">
+      <c r="C18" t="s" s="16">
         <v>307</v>
       </c>
-      <c r="D18" t="s" s="15">
+      <c r="D18" t="s" s="16">
         <v>296</v>
       </c>
     </row>
@@ -3966,7 +4000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="8.0"/>
@@ -3998,185 +4032,199 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="15">
+      <c r="A2" t="s" s="16">
         <v>308</v>
       </c>
-      <c r="B2" t="s" s="15">
+      <c r="B2" t="s" s="16">
         <v>309</v>
       </c>
-      <c r="C2" t="s" s="15">
+      <c r="C2" t="s" s="16">
         <v>310</v>
       </c>
-      <c r="D2" t="s" s="15">
+      <c r="D2" t="s" s="16">
         <v>311</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="15">
+      <c r="A3" t="s" s="16">
         <v>312</v>
       </c>
-      <c r="B3" t="s" s="15">
+      <c r="B3" t="s" s="16">
         <v>309</v>
       </c>
-      <c r="C3" t="s" s="15">
+      <c r="C3" t="s" s="16">
         <v>313</v>
       </c>
-      <c r="D3" t="s" s="15">
+      <c r="D3" t="s" s="16">
         <v>314</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s" s="15">
+      <c r="A4" t="s" s="16">
         <v>315</v>
       </c>
-      <c r="B4" t="s" s="15">
+      <c r="B4" t="s" s="16">
         <v>309</v>
       </c>
-      <c r="C4" t="s" s="15">
+      <c r="C4" t="s" s="16">
         <v>316</v>
       </c>
-      <c r="D4" t="s" s="15">
+      <c r="D4" t="s" s="16">
         <v>317</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s" s="15">
+      <c r="A5" t="s" s="16">
         <v>318</v>
       </c>
-      <c r="B5" t="s" s="15">
+      <c r="B5" t="s" s="16">
         <v>319</v>
       </c>
-      <c r="C5" t="s" s="15">
+      <c r="C5" t="s" s="16">
         <v>320</v>
       </c>
-      <c r="D5" t="s" s="15">
+      <c r="D5" t="s" s="16">
         <v>321</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s" s="15">
+      <c r="A6" t="s" s="16">
         <v>322</v>
       </c>
-      <c r="B6" t="s" s="15">
+      <c r="B6" t="s" s="16">
         <v>323</v>
       </c>
-      <c r="C6" t="s" s="15">
+      <c r="C6" t="s" s="16">
         <v>324</v>
       </c>
-      <c r="D6" t="s" s="15">
+      <c r="D6" t="s" s="16">
         <v>233</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s" s="15">
+      <c r="A7" t="s" s="16">
         <v>325</v>
       </c>
-      <c r="B7" t="s" s="15">
+      <c r="B7" t="s" s="16">
         <v>319</v>
       </c>
-      <c r="C7" t="s" s="15">
+      <c r="C7" t="s" s="16">
         <v>326</v>
       </c>
-      <c r="D7" t="s" s="15">
+      <c r="D7" t="s" s="16">
         <v>327</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="s" s="15">
+      <c r="A8" t="s" s="16">
         <v>328</v>
       </c>
-      <c r="B8" t="s" s="15">
+      <c r="B8" t="s" s="16">
         <v>319</v>
       </c>
-      <c r="C8" t="s" s="15">
+      <c r="C8" t="s" s="16">
         <v>329</v>
       </c>
-      <c r="D8" t="s" s="15">
+      <c r="D8" t="s" s="16">
         <v>113</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="s" s="15">
+      <c r="A9" t="s" s="16">
         <v>330</v>
       </c>
-      <c r="B9" t="s" s="15">
+      <c r="B9" t="s" s="16">
         <v>319</v>
       </c>
-      <c r="C9" t="s" s="15">
+      <c r="C9" t="s" s="16">
         <v>331</v>
       </c>
-      <c r="D9" t="s" s="15">
+      <c r="D9" t="s" s="16">
         <v>257</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="s" s="15">
+      <c r="A10" t="s" s="16">
         <v>332</v>
       </c>
-      <c r="B10" t="s" s="15">
+      <c r="B10" t="s" s="16">
         <v>319</v>
       </c>
-      <c r="C10" t="s" s="15">
+      <c r="C10" t="s" s="16">
         <v>333</v>
       </c>
-      <c r="D10" t="s" s="15">
+      <c r="D10" t="s" s="16">
         <v>67</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="s" s="15">
+      <c r="A11" t="s" s="16">
         <v>334</v>
       </c>
-      <c r="B11" t="s" s="15">
+      <c r="B11" t="s" s="16">
         <v>319</v>
       </c>
-      <c r="C11" t="s" s="15">
+      <c r="C11" t="s" s="16">
         <v>335</v>
       </c>
-      <c r="D11" t="s" s="15">
+      <c r="D11" t="s" s="16">
         <v>336</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="s" s="15">
+      <c r="A12" t="s" s="16">
         <v>337</v>
       </c>
-      <c r="B12" t="s" s="15">
+      <c r="B12" t="s" s="16">
         <v>338</v>
       </c>
-      <c r="C12" t="s" s="15">
+      <c r="C12" t="s" s="16">
         <v>339</v>
       </c>
-      <c r="D12" t="s" s="15">
+      <c r="D12" t="s" s="16">
         <v>233</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="s" s="15">
+      <c r="A13" t="s" s="16">
         <v>340</v>
       </c>
-      <c r="B13" t="s" s="15">
+      <c r="B13" t="s" s="16">
         <v>338</v>
       </c>
-      <c r="C13" t="s" s="15">
+      <c r="C13" t="s" s="16">
         <v>341</v>
       </c>
-      <c r="D13" t="s" s="15">
+      <c r="D13" t="s" s="16">
         <v>342</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="s" s="15">
+      <c r="A14" t="s" s="16">
         <v>348</v>
       </c>
-      <c r="B14" t="s" s="15">
+      <c r="B14" t="s" s="16">
         <v>319</v>
       </c>
-      <c r="C14" t="s" s="15">
+      <c r="C14" t="s" s="16">
         <v>349</v>
       </c>
-      <c r="D14" t="s" s="15">
+      <c r="D14" t="s" s="16">
         <v>15</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="16">
+        <v>356</v>
+      </c>
+      <c r="B15" t="s" s="16">
+        <v>319</v>
+      </c>
+      <c r="C15" t="s" s="16">
+        <v>357</v>
+      </c>
+      <c r="D15" t="s" s="16">
+        <v>257</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: check the page title after a direct load, not after in-app navigation
TC_CNT_009 reached the Company page by clicking the navigation and then waited for the page
title. That is a client side route change: the heading renders while document.title still holds
the previous page's value. On a CI runner the title had not updated after the full 15 second
wait, so the test failed on one run while passing on the runs either side - about one in four.

The title moves to TC_CNT_015, which runs after the page is opened directly, so the title
arrives with the document and there is nothing to race. TC_CNT_009 now checks what its name
says: the page opens from the navigation with the right heading and intro text.

Verified by running the full suite three times on each browser: 57 tests, 0 failures, six runs,
no flakes. Sample reports refreshed to match, and waitForTitleContains removed as unused.
</commit_message>
<xml_diff>
--- a/MBio_Test_Cases.xlsx
+++ b/MBio_Test_Cases.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2466" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3748" uniqueCount="378">
   <si>
     <t>TC_NAV_001</t>
   </si>
@@ -1253,6 +1253,62 @@
   </si>
   <si>
     <t>Chrome 153 and Firefox 156, 1920x1080. Both browsers run the same suite - see docs/sample-reports/</t>
+  </si>
+  <si>
+    <t>Verify the Why MultiBank page opens from the navigation with the correct heading and intro text</t>
+  </si>
+  <si>
+    <t>1. Open https://mb.io/en-AE/
+2. Click 'Company' in the top navigation
+3. Wait for the URL to contain /company
+4. Read the heading and the intro text</t>
+  </si>
+  <si>
+    <t>1. Heading 'Why MultiBank Group?' is visible
+2. Intro text starts with 'For nearly two decades, MultiBank has built a reputation'</t>
+  </si>
+  <si>
+    <t>The brief calls it 'About Us &gt; Why MultiBank'; on the live site it is the 'Company' menu item. The page title is checked in TC_CNT_015 instead - see finding F-15.</t>
+  </si>
+  <si>
+    <t>TC_CNT_015</t>
+  </si>
+  <si>
+    <t>Verify the Why MultiBank page title</t>
+  </si>
+  <si>
+    <t>Expected title: About mb.io | MultiBank Group Exchange Since 2005</t>
+  </si>
+  <si>
+    <t>1. Open /en-AE/company directly
+2. Read the browser page title</t>
+  </si>
+  <si>
+    <t>1. The page title equals 'About mb.io | MultiBank Group Exchange Since 2005'</t>
+  </si>
+  <si>
+    <t>WhyMultiBankTest.verifyPageTitle</t>
+  </si>
+  <si>
+    <t>Checked after opening the page directly, not after clicking through the navigation. A click is a client side route change and the title updates after the content: on a CI runner the title was still the previous page's after a 15 second wait, while the same test passed on the runs either side. See F-15.</t>
+  </si>
+  <si>
+    <t>F-15</t>
+  </si>
+  <si>
+    <t>The page title lags behind the content when a page is reached by clicking the navigation. The Company page heading rendered while document.title still held the previous page's value, and on a CI runner it had not updated after 15 seconds - the same test passed on the runs either side, so it failed about one run in four. The title is now checked in TC_CNT_015 after opening the page directly. Minor, but real: a stale title affects search engines and screen readers.</t>
+  </si>
+  <si>
+    <t>TC_CNT_009, TC_CNT_015</t>
+  </si>
+  <si>
+    <t>2026-09-18 - testng.xml - 57 tests run, 0 failures - three runs on Chrome 153 and three on Firefox 156, no failures and no flakes. 1 further test (TC_NEG_002-KI) is excluded by the 'known-issue' group and fails on purpose.</t>
+  </si>
+  <si>
+    <t>TC_CNT_009, TC_CNT_010, TC_CNT_011, TC_CNT_012, TC_CNT_013, TC_CNT_014, TC_CNT_015</t>
+  </si>
+  <si>
+    <t>7</t>
   </si>
 </sst>
 </file>
@@ -1336,7 +1392,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1363,6 +1419,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+      <alignment wrapText="true" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+      <alignment wrapText="true" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
       <alignment wrapText="true" vertical="top"/>
@@ -1867,7 +1929,7 @@
         <v>345</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>358</v>
+        <v>375</v>
       </c>
     </row>
     <row r="14">
@@ -2046,7 +2108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P34"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="12.0"/>
@@ -2150,1554 +2212,1601 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="16">
+      <c r="A2" t="s" s="18">
         <v>0</v>
       </c>
-      <c r="B2" t="s" s="16">
+      <c r="B2" t="s" s="18">
         <v>1</v>
       </c>
-      <c r="C2" t="s" s="16">
+      <c r="C2" t="s" s="18">
         <v>2</v>
       </c>
-      <c r="D2" t="s" s="16">
+      <c r="D2" t="s" s="18">
         <v>3</v>
       </c>
-      <c r="E2" t="s" s="16">
+      <c r="E2" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F2" t="s" s="16">
+      <c r="F2" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G2" t="s" s="16">
+      <c r="G2" t="s" s="18">
         <v>6</v>
       </c>
-      <c r="H2" t="s" s="16">
+      <c r="H2" t="s" s="18">
         <v>7</v>
       </c>
-      <c r="I2" t="s" s="16">
+      <c r="I2" t="s" s="18">
         <v>8</v>
       </c>
-      <c r="J2" t="s" s="16">
+      <c r="J2" t="s" s="18">
         <v>9</v>
       </c>
-      <c r="K2" t="s" s="16">
+      <c r="K2" t="s" s="18">
         <v>10</v>
       </c>
-      <c r="L2" t="s" s="16">
+      <c r="L2" t="s" s="18">
         <v>11</v>
       </c>
-      <c r="M2" t="s" s="16">
+      <c r="M2" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N2" t="s" s="16">
+      <c r="N2" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P2" t="s" s="16">
+      <c r="P2" t="s" s="18">
         <v>14</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="16">
+      <c r="A3" t="s" s="18">
         <v>15</v>
       </c>
-      <c r="B3" t="s" s="16">
+      <c r="B3" t="s" s="18">
         <v>1</v>
       </c>
-      <c r="C3" t="s" s="16">
+      <c r="C3" t="s" s="18">
         <v>16</v>
       </c>
-      <c r="D3" t="s" s="16">
+      <c r="D3" t="s" s="18">
         <v>17</v>
       </c>
-      <c r="E3" t="s" s="16">
+      <c r="E3" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F3" t="s" s="16">
+      <c r="F3" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G3" t="s" s="16">
+      <c r="G3" t="s" s="18">
         <v>18</v>
       </c>
-      <c r="H3" t="s" s="16">
+      <c r="H3" t="s" s="18">
         <v>19</v>
       </c>
-      <c r="I3" t="s" s="16">
+      <c r="I3" t="s" s="18">
         <v>20</v>
       </c>
-      <c r="J3" t="s" s="16">
+      <c r="J3" t="s" s="18">
         <v>21</v>
       </c>
-      <c r="K3" t="s" s="16">
+      <c r="K3" t="s" s="18">
         <v>22</v>
       </c>
-      <c r="L3" t="s" s="16">
+      <c r="L3" t="s" s="18">
         <v>23</v>
       </c>
-      <c r="M3" t="s" s="16">
+      <c r="M3" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N3" t="s" s="16">
+      <c r="N3" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P3" t="s" s="16">
+      <c r="P3" t="s" s="18">
         <v>347</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s" s="16">
+      <c r="A4" t="s" s="18">
         <v>25</v>
       </c>
-      <c r="B4" t="s" s="16">
+      <c r="B4" t="s" s="18">
         <v>1</v>
       </c>
-      <c r="C4" t="s" s="16">
+      <c r="C4" t="s" s="18">
         <v>16</v>
       </c>
-      <c r="D4" t="s" s="16">
+      <c r="D4" t="s" s="18">
         <v>26</v>
       </c>
-      <c r="E4" t="s" s="16">
+      <c r="E4" t="s" s="18">
         <v>27</v>
       </c>
-      <c r="F4" t="s" s="16">
+      <c r="F4" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G4" t="s" s="16">
+      <c r="G4" t="s" s="18">
         <v>18</v>
       </c>
-      <c r="H4" t="s" s="16">
+      <c r="H4" t="s" s="18">
         <v>28</v>
       </c>
-      <c r="I4" t="s" s="16">
+      <c r="I4" t="s" s="18">
         <v>29</v>
       </c>
-      <c r="J4" t="s" s="16">
+      <c r="J4" t="s" s="18">
         <v>30</v>
       </c>
-      <c r="K4" t="s" s="16">
+      <c r="K4" t="s" s="18">
         <v>31</v>
       </c>
-      <c r="L4" t="s" s="16">
+      <c r="L4" t="s" s="18">
         <v>32</v>
       </c>
-      <c r="M4" t="s" s="16">
+      <c r="M4" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N4" t="s" s="16">
+      <c r="N4" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P4" t="s" s="16">
+      <c r="P4" t="s" s="18">
         <v>33</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s" s="16">
+      <c r="A5" t="s" s="18">
         <v>34</v>
       </c>
-      <c r="B5" t="s" s="16">
+      <c r="B5" t="s" s="18">
         <v>1</v>
       </c>
-      <c r="C5" t="s" s="16">
+      <c r="C5" t="s" s="18">
         <v>16</v>
       </c>
-      <c r="D5" t="s" s="16">
+      <c r="D5" t="s" s="18">
         <v>35</v>
       </c>
-      <c r="E5" t="s" s="16">
+      <c r="E5" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F5" t="s" s="16">
+      <c r="F5" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G5" t="s" s="16">
+      <c r="G5" t="s" s="18">
         <v>18</v>
       </c>
-      <c r="H5" t="s" s="16">
+      <c r="H5" t="s" s="18">
         <v>36</v>
       </c>
-      <c r="I5" t="s" s="16">
+      <c r="I5" t="s" s="18">
         <v>37</v>
       </c>
-      <c r="J5" t="s" s="16">
+      <c r="J5" t="s" s="18">
         <v>38</v>
       </c>
-      <c r="K5" t="s" s="16">
+      <c r="K5" t="s" s="18">
         <v>10</v>
       </c>
-      <c r="L5" t="s" s="16">
+      <c r="L5" t="s" s="18">
         <v>39</v>
       </c>
-      <c r="M5" t="s" s="16">
+      <c r="M5" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N5" t="s" s="16">
+      <c r="N5" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P5" t="s" s="16">
+      <c r="P5" t="s" s="18">
         <v>40</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s" s="16">
+      <c r="A6" t="s" s="18">
         <v>41</v>
       </c>
-      <c r="B6" t="s" s="16">
+      <c r="B6" t="s" s="18">
         <v>1</v>
       </c>
-      <c r="C6" t="s" s="16">
+      <c r="C6" t="s" s="18">
         <v>42</v>
       </c>
-      <c r="D6" t="s" s="16">
+      <c r="D6" t="s" s="18">
         <v>43</v>
       </c>
-      <c r="E6" t="s" s="16">
+      <c r="E6" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F6" t="s" s="16">
+      <c r="F6" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G6" t="s" s="16">
+      <c r="G6" t="s" s="18">
         <v>44</v>
       </c>
-      <c r="H6" t="s" s="16">
+      <c r="H6" t="s" s="18">
         <v>45</v>
       </c>
-      <c r="I6" t="s" s="16">
+      <c r="I6" t="s" s="18">
         <v>46</v>
       </c>
-      <c r="J6" t="s" s="16">
+      <c r="J6" t="s" s="18">
         <v>47</v>
       </c>
-      <c r="K6" t="s" s="16">
+      <c r="K6" t="s" s="18">
         <v>22</v>
       </c>
-      <c r="L6" t="s" s="16">
+      <c r="L6" t="s" s="18">
         <v>48</v>
       </c>
-      <c r="M6" t="s" s="16">
+      <c r="M6" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N6" t="s" s="16">
+      <c r="N6" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P6" t="s" s="16">
+      <c r="P6" t="s" s="18">
         <v>49</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s" s="16">
+      <c r="A7" t="s" s="18">
         <v>50</v>
       </c>
-      <c r="B7" t="s" s="16">
+      <c r="B7" t="s" s="18">
         <v>1</v>
       </c>
-      <c r="C7" t="s" s="16">
+      <c r="C7" t="s" s="18">
         <v>16</v>
       </c>
-      <c r="D7" t="s" s="16">
+      <c r="D7" t="s" s="18">
         <v>51</v>
       </c>
-      <c r="E7" t="s" s="16">
+      <c r="E7" t="s" s="18">
         <v>27</v>
       </c>
-      <c r="F7" t="s" s="16">
+      <c r="F7" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G7" t="s" s="16">
+      <c r="G7" t="s" s="18">
         <v>18</v>
       </c>
-      <c r="H7" t="s" s="16">
+      <c r="H7" t="s" s="18">
         <v>52</v>
       </c>
-      <c r="I7" t="s" s="16">
+      <c r="I7" t="s" s="18">
         <v>53</v>
       </c>
-      <c r="J7" t="s" s="16">
+      <c r="J7" t="s" s="18">
         <v>54</v>
       </c>
-      <c r="K7" t="s" s="16">
+      <c r="K7" t="s" s="18">
         <v>31</v>
       </c>
-      <c r="L7" t="s" s="16">
+      <c r="L7" t="s" s="18">
         <v>55</v>
       </c>
-      <c r="M7" t="s" s="16">
+      <c r="M7" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N7" t="s" s="16">
+      <c r="N7" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P7" t="s" s="16">
+      <c r="P7" t="s" s="18">
         <v>13</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="s" s="16">
+      <c r="A8" t="s" s="18">
         <v>56</v>
       </c>
-      <c r="B8" t="s" s="16">
+      <c r="B8" t="s" s="18">
         <v>57</v>
       </c>
-      <c r="C8" t="s" s="16">
+      <c r="C8" t="s" s="18">
         <v>58</v>
       </c>
-      <c r="D8" t="s" s="16">
+      <c r="D8" t="s" s="18">
         <v>59</v>
       </c>
-      <c r="E8" t="s" s="16">
+      <c r="E8" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F8" t="s" s="16">
+      <c r="F8" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G8" t="s" s="16">
+      <c r="G8" t="s" s="18">
         <v>60</v>
       </c>
-      <c r="H8" t="s" s="16">
+      <c r="H8" t="s" s="18">
         <v>61</v>
       </c>
-      <c r="I8" t="s" s="16">
+      <c r="I8" t="s" s="18">
         <v>62</v>
       </c>
-      <c r="J8" t="s" s="16">
+      <c r="J8" t="s" s="18">
         <v>63</v>
       </c>
-      <c r="K8" t="s" s="16">
+      <c r="K8" t="s" s="18">
         <v>64</v>
       </c>
-      <c r="L8" t="s" s="16">
+      <c r="L8" t="s" s="18">
         <v>65</v>
       </c>
-      <c r="M8" t="s" s="16">
+      <c r="M8" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N8" t="s" s="16">
+      <c r="N8" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P8" t="s" s="16">
+      <c r="P8" t="s" s="18">
         <v>66</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="s" s="16">
+      <c r="A9" t="s" s="18">
         <v>67</v>
       </c>
-      <c r="B9" t="s" s="16">
+      <c r="B9" t="s" s="18">
         <v>57</v>
       </c>
-      <c r="C9" t="s" s="16">
+      <c r="C9" t="s" s="18">
         <v>58</v>
       </c>
-      <c r="D9" t="s" s="16">
+      <c r="D9" t="s" s="18">
         <v>68</v>
       </c>
-      <c r="E9" t="s" s="16">
+      <c r="E9" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F9" t="s" s="16">
+      <c r="F9" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G9" t="s" s="16">
+      <c r="G9" t="s" s="18">
         <v>69</v>
       </c>
-      <c r="H9" t="s" s="16">
+      <c r="H9" t="s" s="18">
         <v>70</v>
       </c>
-      <c r="I9" t="s" s="16">
+      <c r="I9" t="s" s="18">
         <v>71</v>
       </c>
-      <c r="J9" t="s" s="16">
+      <c r="J9" t="s" s="18">
         <v>72</v>
       </c>
-      <c r="K9" t="s" s="16">
+      <c r="K9" t="s" s="18">
         <v>64</v>
       </c>
-      <c r="L9" t="s" s="16">
+      <c r="L9" t="s" s="18">
         <v>73</v>
       </c>
-      <c r="M9" t="s" s="16">
+      <c r="M9" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N9" t="s" s="16">
+      <c r="N9" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P9" t="s" s="16">
+      <c r="P9" t="s" s="18">
         <v>74</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="s" s="16">
+      <c r="A10" t="s" s="18">
         <v>75</v>
       </c>
-      <c r="B10" t="s" s="16">
+      <c r="B10" t="s" s="18">
         <v>57</v>
       </c>
-      <c r="C10" t="s" s="16">
+      <c r="C10" t="s" s="18">
         <v>76</v>
       </c>
-      <c r="D10" t="s" s="16">
+      <c r="D10" t="s" s="18">
         <v>77</v>
       </c>
-      <c r="E10" t="s" s="16">
+      <c r="E10" t="s" s="18">
         <v>27</v>
       </c>
-      <c r="F10" t="s" s="16">
+      <c r="F10" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G10" t="s" s="16">
+      <c r="G10" t="s" s="18">
         <v>78</v>
       </c>
-      <c r="H10" t="s" s="16">
+      <c r="H10" t="s" s="18">
         <v>79</v>
       </c>
-      <c r="I10" t="s" s="16">
+      <c r="I10" t="s" s="18">
         <v>80</v>
       </c>
-      <c r="J10" t="s" s="16">
+      <c r="J10" t="s" s="18">
         <v>81</v>
       </c>
-      <c r="K10" t="s" s="16">
+      <c r="K10" t="s" s="18">
         <v>82</v>
       </c>
-      <c r="L10" t="s" s="16">
+      <c r="L10" t="s" s="18">
         <v>83</v>
       </c>
-      <c r="M10" t="s" s="16">
+      <c r="M10" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N10" t="s" s="16">
+      <c r="N10" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P10" t="s" s="16">
+      <c r="P10" t="s" s="18">
         <v>84</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="s" s="16">
+      <c r="A11" t="s" s="18">
         <v>85</v>
       </c>
-      <c r="B11" t="s" s="16">
+      <c r="B11" t="s" s="18">
         <v>57</v>
       </c>
-      <c r="C11" t="s" s="16">
+      <c r="C11" t="s" s="18">
         <v>76</v>
       </c>
-      <c r="D11" t="s" s="16">
+      <c r="D11" t="s" s="18">
         <v>86</v>
       </c>
-      <c r="E11" t="s" s="16">
+      <c r="E11" t="s" s="18">
         <v>27</v>
       </c>
-      <c r="F11" t="s" s="16">
+      <c r="F11" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G11" t="s" s="16">
+      <c r="G11" t="s" s="18">
         <v>69</v>
       </c>
-      <c r="H11" t="s" s="16">
+      <c r="H11" t="s" s="18">
         <v>87</v>
       </c>
-      <c r="I11" t="s" s="16">
+      <c r="I11" t="s" s="18">
         <v>88</v>
       </c>
-      <c r="J11" t="s" s="16">
+      <c r="J11" t="s" s="18">
         <v>89</v>
       </c>
-      <c r="K11" t="s" s="16">
+      <c r="K11" t="s" s="18">
         <v>82</v>
       </c>
-      <c r="L11" t="s" s="16">
+      <c r="L11" t="s" s="18">
         <v>90</v>
       </c>
-      <c r="M11" t="s" s="16">
+      <c r="M11" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N11" t="s" s="16">
+      <c r="N11" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P11" t="s" s="16">
+      <c r="P11" t="s" s="18">
         <v>91</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="s" s="16">
+      <c r="A12" t="s" s="18">
         <v>92</v>
       </c>
-      <c r="B12" t="s" s="16">
+      <c r="B12" t="s" s="18">
         <v>57</v>
       </c>
-      <c r="C12" t="s" s="16">
+      <c r="C12" t="s" s="18">
         <v>76</v>
       </c>
-      <c r="D12" t="s" s="16">
+      <c r="D12" t="s" s="18">
         <v>93</v>
       </c>
-      <c r="E12" t="s" s="16">
+      <c r="E12" t="s" s="18">
         <v>27</v>
       </c>
-      <c r="F12" t="s" s="16">
+      <c r="F12" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G12" t="s" s="16">
+      <c r="G12" t="s" s="18">
         <v>69</v>
       </c>
-      <c r="H12" t="s" s="16">
+      <c r="H12" t="s" s="18">
         <v>87</v>
       </c>
-      <c r="I12" t="s" s="16">
+      <c r="I12" t="s" s="18">
         <v>94</v>
       </c>
-      <c r="J12" t="s" s="16">
+      <c r="J12" t="s" s="18">
         <v>95</v>
       </c>
-      <c r="K12" t="s" s="16">
+      <c r="K12" t="s" s="18">
         <v>82</v>
       </c>
-      <c r="L12" t="s" s="16">
+      <c r="L12" t="s" s="18">
         <v>96</v>
       </c>
-      <c r="M12" t="s" s="16">
+      <c r="M12" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N12" t="s" s="16">
+      <c r="N12" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P12" t="s" s="16">
+      <c r="P12" t="s" s="18">
         <v>97</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="s" s="16">
+      <c r="A13" t="s" s="18">
         <v>98</v>
       </c>
-      <c r="B13" t="s" s="16">
+      <c r="B13" t="s" s="18">
         <v>57</v>
       </c>
-      <c r="C13" t="s" s="16">
+      <c r="C13" t="s" s="18">
         <v>99</v>
       </c>
-      <c r="D13" t="s" s="16">
+      <c r="D13" t="s" s="18">
         <v>100</v>
       </c>
-      <c r="E13" t="s" s="16">
+      <c r="E13" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F13" t="s" s="16">
+      <c r="F13" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G13" t="s" s="16">
+      <c r="G13" t="s" s="18">
         <v>69</v>
       </c>
-      <c r="H13" t="s" s="16">
+      <c r="H13" t="s" s="18">
         <v>101</v>
       </c>
-      <c r="I13" t="s" s="16">
+      <c r="I13" t="s" s="18">
         <v>102</v>
       </c>
-      <c r="J13" t="s" s="16">
+      <c r="J13" t="s" s="18">
         <v>103</v>
       </c>
-      <c r="K13" t="s" s="16">
+      <c r="K13" t="s" s="18">
         <v>64</v>
       </c>
-      <c r="L13" t="s" s="16">
+      <c r="L13" t="s" s="18">
         <v>104</v>
       </c>
-      <c r="M13" t="s" s="16">
+      <c r="M13" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N13" t="s" s="16">
+      <c r="N13" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P13" t="s" s="16">
+      <c r="P13" t="s" s="18">
         <v>105</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="s" s="16">
+      <c r="A14" t="s" s="18">
         <v>106</v>
       </c>
-      <c r="B14" t="s" s="16">
+      <c r="B14" t="s" s="18">
         <v>57</v>
       </c>
-      <c r="C14" t="s" s="16">
+      <c r="C14" t="s" s="18">
         <v>76</v>
       </c>
-      <c r="D14" t="s" s="16">
+      <c r="D14" t="s" s="18">
         <v>107</v>
       </c>
-      <c r="E14" t="s" s="16">
+      <c r="E14" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F14" t="s" s="16">
+      <c r="F14" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G14" t="s" s="16">
+      <c r="G14" t="s" s="18">
         <v>108</v>
       </c>
-      <c r="H14" t="s" s="16">
+      <c r="H14" t="s" s="18">
         <v>79</v>
       </c>
-      <c r="I14" t="s" s="16">
+      <c r="I14" t="s" s="18">
         <v>109</v>
       </c>
-      <c r="J14" t="s" s="16">
+      <c r="J14" t="s" s="18">
         <v>110</v>
       </c>
-      <c r="K14" t="s" s="16">
+      <c r="K14" t="s" s="18">
         <v>111</v>
       </c>
-      <c r="L14" t="s" s="16">
+      <c r="L14" t="s" s="18">
         <v>112</v>
       </c>
-      <c r="M14" t="s" s="16">
+      <c r="M14" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N14" t="s" s="16">
+      <c r="N14" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P14" t="s" s="16">
+      <c r="P14" t="s" s="18">
         <v>13</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="s" s="16">
+      <c r="A15" t="s" s="18">
         <v>113</v>
       </c>
-      <c r="B15" t="s" s="16">
+      <c r="B15" t="s" s="18">
         <v>57</v>
       </c>
-      <c r="C15" t="s" s="16">
+      <c r="C15" t="s" s="18">
         <v>76</v>
       </c>
-      <c r="D15" t="s" s="16">
+      <c r="D15" t="s" s="18">
         <v>114</v>
       </c>
-      <c r="E15" t="s" s="16">
+      <c r="E15" t="s" s="18">
         <v>27</v>
       </c>
-      <c r="F15" t="s" s="16">
+      <c r="F15" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G15" t="s" s="16">
+      <c r="G15" t="s" s="18">
         <v>108</v>
       </c>
-      <c r="H15" t="s" s="16">
+      <c r="H15" t="s" s="18">
         <v>79</v>
       </c>
-      <c r="I15" t="s" s="16">
+      <c r="I15" t="s" s="18">
         <v>115</v>
       </c>
-      <c r="J15" t="s" s="16">
+      <c r="J15" t="s" s="18">
         <v>116</v>
       </c>
-      <c r="K15" t="s" s="16">
+      <c r="K15" t="s" s="18">
         <v>117</v>
       </c>
-      <c r="L15" t="s" s="16">
+      <c r="L15" t="s" s="18">
         <v>118</v>
       </c>
-      <c r="M15" t="s" s="16">
+      <c r="M15" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N15" t="s" s="16">
+      <c r="N15" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P15" t="s" s="16">
+      <c r="P15" t="s" s="18">
         <v>119</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="s" s="16">
+      <c r="A16" t="s" s="18">
         <v>120</v>
       </c>
-      <c r="B16" t="s" s="16">
+      <c r="B16" t="s" s="18">
         <v>57</v>
       </c>
-      <c r="C16" t="s" s="16">
+      <c r="C16" t="s" s="18">
         <v>121</v>
       </c>
-      <c r="D16" t="s" s="16">
+      <c r="D16" t="s" s="18">
         <v>122</v>
       </c>
-      <c r="E16" t="s" s="16">
+      <c r="E16" t="s" s="18">
         <v>27</v>
       </c>
-      <c r="F16" t="s" s="16">
+      <c r="F16" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G16" t="s" s="16">
+      <c r="G16" t="s" s="18">
         <v>108</v>
       </c>
-      <c r="H16" t="s" s="16">
+      <c r="H16" t="s" s="18">
         <v>123</v>
       </c>
-      <c r="I16" t="s" s="16">
+      <c r="I16" t="s" s="18">
         <v>124</v>
       </c>
-      <c r="J16" t="s" s="16">
+      <c r="J16" t="s" s="18">
         <v>125</v>
       </c>
-      <c r="K16" t="s" s="16">
+      <c r="K16" t="s" s="18">
         <v>117</v>
       </c>
-      <c r="L16" t="s" s="16">
+      <c r="L16" t="s" s="18">
         <v>126</v>
       </c>
-      <c r="M16" t="s" s="16">
+      <c r="M16" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N16" t="s" s="16">
+      <c r="N16" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P16" t="s" s="16">
+      <c r="P16" t="s" s="18">
         <v>127</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="s" s="16">
+      <c r="A17" t="s" s="18">
         <v>128</v>
       </c>
-      <c r="B17" t="s" s="16">
+      <c r="B17" t="s" s="18">
         <v>129</v>
       </c>
-      <c r="C17" t="s" s="16">
+      <c r="C17" t="s" s="18">
         <v>130</v>
       </c>
-      <c r="D17" t="s" s="16">
+      <c r="D17" t="s" s="18">
         <v>131</v>
       </c>
-      <c r="E17" t="s" s="16">
+      <c r="E17" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F17" t="s" s="16">
+      <c r="F17" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G17" t="s" s="16">
+      <c r="G17" t="s" s="18">
         <v>18</v>
       </c>
-      <c r="H17" t="s" s="16">
+      <c r="H17" t="s" s="18">
         <v>132</v>
       </c>
-      <c r="I17" t="s" s="16">
+      <c r="I17" t="s" s="18">
         <v>133</v>
       </c>
-      <c r="J17" t="s" s="16">
+      <c r="J17" t="s" s="18">
         <v>134</v>
       </c>
-      <c r="K17" t="s" s="16">
+      <c r="K17" t="s" s="18">
         <v>135</v>
       </c>
-      <c r="L17" t="s" s="16">
+      <c r="L17" t="s" s="18">
         <v>136</v>
       </c>
-      <c r="M17" t="s" s="16">
+      <c r="M17" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N17" t="s" s="16">
+      <c r="N17" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P17" t="s" s="16">
+      <c r="P17" t="s" s="18">
         <v>137</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="s" s="16">
+      <c r="A18" t="s" s="18">
         <v>138</v>
       </c>
-      <c r="B18" t="s" s="16">
+      <c r="B18" t="s" s="18">
         <v>129</v>
       </c>
-      <c r="C18" t="s" s="16">
+      <c r="C18" t="s" s="18">
         <v>139</v>
       </c>
-      <c r="D18" t="s" s="16">
+      <c r="D18" t="s" s="18">
         <v>140</v>
       </c>
-      <c r="E18" t="s" s="16">
+      <c r="E18" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F18" t="s" s="16">
+      <c r="F18" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G18" t="s" s="16">
+      <c r="G18" t="s" s="18">
         <v>18</v>
       </c>
-      <c r="H18" t="s" s="16">
+      <c r="H18" t="s" s="18">
         <v>141</v>
       </c>
-      <c r="I18" t="s" s="16">
+      <c r="I18" t="s" s="18">
         <v>142</v>
       </c>
-      <c r="J18" t="s" s="16">
+      <c r="J18" t="s" s="18">
         <v>143</v>
       </c>
-      <c r="K18" t="s" s="16">
+      <c r="K18" t="s" s="18">
         <v>144</v>
       </c>
-      <c r="L18" t="s" s="16">
+      <c r="L18" t="s" s="18">
         <v>145</v>
       </c>
-      <c r="M18" t="s" s="16">
+      <c r="M18" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N18" t="s" s="16">
+      <c r="N18" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P18" t="s" s="16">
+      <c r="P18" t="s" s="18">
         <v>13</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="s" s="16">
+      <c r="A19" t="s" s="18">
         <v>146</v>
       </c>
-      <c r="B19" t="s" s="16">
+      <c r="B19" t="s" s="18">
         <v>129</v>
       </c>
-      <c r="C19" t="s" s="16">
+      <c r="C19" t="s" s="18">
         <v>139</v>
       </c>
-      <c r="D19" t="s" s="16">
+      <c r="D19" t="s" s="18">
         <v>147</v>
       </c>
-      <c r="E19" t="s" s="16">
+      <c r="E19" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F19" t="s" s="16">
+      <c r="F19" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G19" t="s" s="16">
+      <c r="G19" t="s" s="18">
         <v>148</v>
       </c>
-      <c r="H19" t="s" s="16">
+      <c r="H19" t="s" s="18">
         <v>149</v>
       </c>
-      <c r="I19" t="s" s="16">
+      <c r="I19" t="s" s="18">
         <v>150</v>
       </c>
-      <c r="J19" t="s" s="16">
+      <c r="J19" t="s" s="18">
         <v>151</v>
       </c>
-      <c r="K19" t="s" s="16">
+      <c r="K19" t="s" s="18">
         <v>111</v>
       </c>
-      <c r="L19" t="s" s="16">
+      <c r="L19" t="s" s="18">
         <v>152</v>
       </c>
-      <c r="M19" t="s" s="16">
+      <c r="M19" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N19" t="s" s="16">
+      <c r="N19" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P19" t="s" s="16">
+      <c r="P19" t="s" s="18">
         <v>153</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="s" s="16">
+      <c r="A20" t="s" s="18">
         <v>154</v>
       </c>
-      <c r="B20" t="s" s="16">
+      <c r="B20" t="s" s="18">
         <v>129</v>
       </c>
-      <c r="C20" t="s" s="16">
+      <c r="C20" t="s" s="18">
         <v>139</v>
       </c>
-      <c r="D20" t="s" s="16">
+      <c r="D20" t="s" s="18">
         <v>155</v>
       </c>
-      <c r="E20" t="s" s="16">
+      <c r="E20" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F20" t="s" s="16">
+      <c r="F20" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G20" t="s" s="16">
+      <c r="G20" t="s" s="18">
         <v>148</v>
       </c>
-      <c r="H20" t="s" s="16">
+      <c r="H20" t="s" s="18">
         <v>156</v>
       </c>
-      <c r="I20" t="s" s="16">
+      <c r="I20" t="s" s="18">
         <v>157</v>
       </c>
-      <c r="J20" t="s" s="16">
+      <c r="J20" t="s" s="18">
         <v>158</v>
       </c>
-      <c r="K20" t="s" s="16">
+      <c r="K20" t="s" s="18">
         <v>111</v>
       </c>
-      <c r="L20" t="s" s="16">
+      <c r="L20" t="s" s="18">
         <v>159</v>
       </c>
-      <c r="M20" t="s" s="16">
+      <c r="M20" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N20" t="s" s="16">
+      <c r="N20" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P20" t="s" s="16">
+      <c r="P20" t="s" s="18">
         <v>160</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="s" s="16">
+      <c r="A21" t="s" s="18">
         <v>161</v>
       </c>
-      <c r="B21" t="s" s="16">
+      <c r="B21" t="s" s="18">
         <v>129</v>
       </c>
-      <c r="C21" t="s" s="16">
+      <c r="C21" t="s" s="18">
         <v>139</v>
       </c>
-      <c r="D21" t="s" s="16">
+      <c r="D21" t="s" s="18">
         <v>162</v>
       </c>
-      <c r="E21" t="s" s="16">
+      <c r="E21" t="s" s="18">
         <v>27</v>
       </c>
-      <c r="F21" t="s" s="16">
+      <c r="F21" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G21" t="s" s="16">
+      <c r="G21" t="s" s="18">
         <v>18</v>
       </c>
-      <c r="H21" t="s" s="16">
+      <c r="H21" t="s" s="18">
         <v>163</v>
       </c>
-      <c r="I21" t="s" s="16">
+      <c r="I21" t="s" s="18">
         <v>164</v>
       </c>
-      <c r="J21" t="s" s="16">
+      <c r="J21" t="s" s="18">
         <v>165</v>
       </c>
-      <c r="K21" t="s" s="16">
+      <c r="K21" t="s" s="18">
         <v>166</v>
       </c>
-      <c r="L21" t="s" s="16">
+      <c r="L21" t="s" s="18">
         <v>167</v>
       </c>
-      <c r="M21" t="s" s="16">
+      <c r="M21" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N21" t="s" s="16">
+      <c r="N21" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P21" t="s" s="16">
+      <c r="P21" t="s" s="18">
         <v>168</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="s" s="16">
+      <c r="A22" t="s" s="18">
         <v>169</v>
       </c>
-      <c r="B22" t="s" s="16">
+      <c r="B22" t="s" s="18">
         <v>129</v>
       </c>
-      <c r="C22" t="s" s="16">
+      <c r="C22" t="s" s="18">
         <v>170</v>
       </c>
-      <c r="D22" t="s" s="16">
-        <v>171</v>
-      </c>
-      <c r="E22" t="s" s="16">
+      <c r="D22" t="s" s="18">
+        <v>361</v>
+      </c>
+      <c r="E22" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F22" t="s" s="16">
+      <c r="F22" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G22" t="s" s="16">
+      <c r="G22" t="s" s="18">
         <v>18</v>
       </c>
-      <c r="H22" t="s" s="16">
+      <c r="H22" t="s" s="18">
         <v>172</v>
       </c>
-      <c r="I22" t="s" s="16">
-        <v>173</v>
-      </c>
-      <c r="J22" t="s" s="16">
-        <v>174</v>
-      </c>
-      <c r="K22" t="s" s="16">
+      <c r="I22" t="s" s="18">
+        <v>362</v>
+      </c>
+      <c r="J22" t="s" s="18">
+        <v>363</v>
+      </c>
+      <c r="K22" t="s" s="18">
         <v>144</v>
       </c>
-      <c r="L22" t="s" s="16">
+      <c r="L22" t="s" s="18">
         <v>175</v>
       </c>
-      <c r="M22" t="s" s="16">
+      <c r="M22" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N22" t="s" s="16">
+      <c r="N22" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P22" t="s" s="16">
-        <v>176</v>
+      <c r="P22" t="s" s="18">
+        <v>364</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="s" s="16">
+      <c r="A23" t="s" s="18">
         <v>177</v>
       </c>
-      <c r="B23" t="s" s="16">
+      <c r="B23" t="s" s="18">
         <v>129</v>
       </c>
-      <c r="C23" t="s" s="16">
+      <c r="C23" t="s" s="18">
         <v>170</v>
       </c>
-      <c r="D23" t="s" s="16">
+      <c r="D23" t="s" s="18">
         <v>178</v>
       </c>
-      <c r="E23" t="s" s="16">
+      <c r="E23" t="s" s="18">
         <v>27</v>
       </c>
-      <c r="F23" t="s" s="16">
+      <c r="F23" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G23" t="s" s="16">
+      <c r="G23" t="s" s="18">
         <v>179</v>
       </c>
-      <c r="H23" t="s" s="16">
+      <c r="H23" t="s" s="18">
         <v>180</v>
       </c>
-      <c r="I23" t="s" s="16">
+      <c r="I23" t="s" s="18">
         <v>181</v>
       </c>
-      <c r="J23" t="s" s="16">
+      <c r="J23" t="s" s="18">
         <v>182</v>
       </c>
-      <c r="K23" t="s" s="16">
+      <c r="K23" t="s" s="18">
         <v>183</v>
       </c>
-      <c r="L23" t="s" s="16">
+      <c r="L23" t="s" s="18">
         <v>184</v>
       </c>
-      <c r="M23" t="s" s="16">
+      <c r="M23" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N23" t="s" s="16">
+      <c r="N23" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P23" t="s" s="16">
+      <c r="P23" t="s" s="18">
         <v>185</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="s" s="16">
+      <c r="A24" t="s" s="18">
         <v>186</v>
       </c>
-      <c r="B24" t="s" s="16">
+      <c r="B24" t="s" s="18">
         <v>129</v>
       </c>
-      <c r="C24" t="s" s="16">
+      <c r="C24" t="s" s="18">
         <v>170</v>
       </c>
-      <c r="D24" t="s" s="16">
+      <c r="D24" t="s" s="18">
         <v>187</v>
       </c>
-      <c r="E24" t="s" s="16">
+      <c r="E24" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F24" t="s" s="16">
+      <c r="F24" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G24" t="s" s="16">
+      <c r="G24" t="s" s="18">
         <v>179</v>
       </c>
-      <c r="H24" t="s" s="16">
+      <c r="H24" t="s" s="18">
         <v>188</v>
       </c>
-      <c r="I24" t="s" s="16">
+      <c r="I24" t="s" s="18">
         <v>189</v>
       </c>
-      <c r="J24" t="s" s="16">
+      <c r="J24" t="s" s="18">
         <v>190</v>
       </c>
-      <c r="K24" t="s" s="16">
+      <c r="K24" t="s" s="18">
         <v>135</v>
       </c>
-      <c r="L24" t="s" s="16">
+      <c r="L24" t="s" s="18">
         <v>191</v>
       </c>
-      <c r="M24" t="s" s="16">
+      <c r="M24" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N24" t="s" s="16">
+      <c r="N24" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P24" t="s" s="16">
+      <c r="P24" t="s" s="18">
         <v>13</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="s" s="16">
+      <c r="A25" t="s" s="18">
         <v>192</v>
       </c>
-      <c r="B25" t="s" s="16">
+      <c r="B25" t="s" s="18">
         <v>129</v>
       </c>
-      <c r="C25" t="s" s="16">
+      <c r="C25" t="s" s="18">
         <v>170</v>
       </c>
-      <c r="D25" t="s" s="16">
+      <c r="D25" t="s" s="18">
         <v>193</v>
       </c>
-      <c r="E25" t="s" s="16">
+      <c r="E25" t="s" s="18">
         <v>27</v>
       </c>
-      <c r="F25" t="s" s="16">
+      <c r="F25" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G25" t="s" s="16">
+      <c r="G25" t="s" s="18">
         <v>179</v>
       </c>
-      <c r="H25" t="s" s="16">
+      <c r="H25" t="s" s="18">
         <v>194</v>
       </c>
-      <c r="I25" t="s" s="16">
+      <c r="I25" t="s" s="18">
         <v>195</v>
       </c>
-      <c r="J25" t="s" s="16">
+      <c r="J25" t="s" s="18">
         <v>196</v>
       </c>
-      <c r="K25" t="s" s="16">
+      <c r="K25" t="s" s="18">
         <v>166</v>
       </c>
-      <c r="L25" t="s" s="16">
+      <c r="L25" t="s" s="18">
         <v>197</v>
       </c>
-      <c r="M25" t="s" s="16">
+      <c r="M25" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N25" t="s" s="16">
+      <c r="N25" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P25" t="s" s="16">
+      <c r="P25" t="s" s="18">
         <v>13</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="s" s="16">
+      <c r="A26" t="s" s="18">
         <v>198</v>
       </c>
-      <c r="B26" t="s" s="16">
+      <c r="B26" t="s" s="18">
         <v>129</v>
       </c>
-      <c r="C26" t="s" s="16">
+      <c r="C26" t="s" s="18">
         <v>170</v>
       </c>
-      <c r="D26" t="s" s="16">
+      <c r="D26" t="s" s="18">
         <v>199</v>
       </c>
-      <c r="E26" t="s" s="16">
+      <c r="E26" t="s" s="18">
         <v>27</v>
       </c>
-      <c r="F26" t="s" s="16">
+      <c r="F26" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G26" t="s" s="16">
+      <c r="G26" t="s" s="18">
         <v>179</v>
       </c>
-      <c r="H26" t="s" s="16">
+      <c r="H26" t="s" s="18">
         <v>200</v>
       </c>
-      <c r="I26" t="s" s="16">
+      <c r="I26" t="s" s="18">
         <v>201</v>
       </c>
-      <c r="J26" t="s" s="16">
+      <c r="J26" t="s" s="18">
         <v>202</v>
       </c>
-      <c r="K26" t="s" s="16">
+      <c r="K26" t="s" s="18">
         <v>166</v>
       </c>
-      <c r="L26" t="s" s="16">
+      <c r="L26" t="s" s="18">
         <v>203</v>
       </c>
-      <c r="M26" t="s" s="16">
+      <c r="M26" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N26" t="s" s="16">
+      <c r="N26" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P26" t="s" s="16">
+      <c r="P26" t="s" s="18">
         <v>204</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="s" s="16">
+      <c r="A27" t="s" s="18">
         <v>205</v>
       </c>
-      <c r="B27" t="s" s="16">
+      <c r="B27" t="s" s="18">
         <v>129</v>
       </c>
-      <c r="C27" t="s" s="16">
+      <c r="C27" t="s" s="18">
         <v>170</v>
       </c>
-      <c r="D27" t="s" s="16">
+      <c r="D27" t="s" s="18">
         <v>206</v>
       </c>
-      <c r="E27" t="s" s="16">
+      <c r="E27" t="s" s="18">
         <v>27</v>
       </c>
-      <c r="F27" t="s" s="16">
+      <c r="F27" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G27" t="s" s="16">
+      <c r="G27" t="s" s="18">
         <v>179</v>
       </c>
-      <c r="H27" t="s" s="16">
+      <c r="H27" t="s" s="18">
         <v>207</v>
       </c>
-      <c r="I27" t="s" s="16">
+      <c r="I27" t="s" s="18">
         <v>208</v>
       </c>
-      <c r="J27" t="s" s="16">
+      <c r="J27" t="s" s="18">
         <v>209</v>
       </c>
-      <c r="K27" t="s" s="16">
+      <c r="K27" t="s" s="18">
         <v>166</v>
       </c>
-      <c r="L27" t="s" s="16">
+      <c r="L27" t="s" s="18">
         <v>210</v>
       </c>
-      <c r="M27" t="s" s="16">
+      <c r="M27" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N27" t="s" s="16">
+      <c r="N27" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P27" t="s" s="16">
+      <c r="P27" t="s" s="18">
         <v>211</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="s" s="16">
+      <c r="A28" t="s" s="18">
         <v>212</v>
       </c>
-      <c r="B28" t="s" s="16">
+      <c r="B28" t="s" s="18">
         <v>213</v>
       </c>
-      <c r="C28" t="s" s="16">
+      <c r="C28" t="s" s="18">
         <v>214</v>
       </c>
-      <c r="D28" t="s" s="16">
+      <c r="D28" t="s" s="18">
         <v>215</v>
       </c>
-      <c r="E28" t="s" s="16">
+      <c r="E28" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F28" t="s" s="16">
+      <c r="F28" t="s" s="18">
         <v>216</v>
       </c>
-      <c r="G28" t="s" s="16">
+      <c r="G28" t="s" s="18">
         <v>217</v>
       </c>
-      <c r="H28" t="s" s="16">
+      <c r="H28" t="s" s="18">
         <v>218</v>
       </c>
-      <c r="I28" t="s" s="16">
+      <c r="I28" t="s" s="18">
         <v>219</v>
       </c>
-      <c r="J28" t="s" s="16">
+      <c r="J28" t="s" s="18">
         <v>220</v>
       </c>
-      <c r="K28" t="s" s="16">
+      <c r="K28" t="s" s="18">
         <v>221</v>
       </c>
-      <c r="L28" t="s" s="16">
+      <c r="L28" t="s" s="18">
         <v>222</v>
       </c>
-      <c r="M28" t="s" s="16">
+      <c r="M28" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N28" t="s" s="16">
+      <c r="N28" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P28" t="s" s="16">
+      <c r="P28" t="s" s="18">
         <v>223</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="s" s="16">
+      <c r="A29" t="s" s="18">
         <v>224</v>
       </c>
-      <c r="B29" t="s" s="16">
+      <c r="B29" t="s" s="18">
         <v>213</v>
       </c>
-      <c r="C29" t="s" s="16">
+      <c r="C29" t="s" s="18">
         <v>214</v>
       </c>
-      <c r="D29" t="s" s="16">
+      <c r="D29" t="s" s="18">
         <v>225</v>
       </c>
-      <c r="E29" t="s" s="16">
+      <c r="E29" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F29" t="s" s="16">
+      <c r="F29" t="s" s="18">
         <v>216</v>
       </c>
-      <c r="G29" t="s" s="16">
+      <c r="G29" t="s" s="18">
         <v>226</v>
       </c>
-      <c r="H29" t="s" s="16">
+      <c r="H29" t="s" s="18">
         <v>227</v>
       </c>
-      <c r="I29" t="s" s="16">
+      <c r="I29" t="s" s="18">
         <v>228</v>
       </c>
-      <c r="J29" t="s" s="16">
+      <c r="J29" t="s" s="18">
         <v>229</v>
       </c>
-      <c r="K29" t="s" s="16">
+      <c r="K29" t="s" s="18">
         <v>230</v>
       </c>
-      <c r="L29" t="s" s="16">
+      <c r="L29" t="s" s="18">
         <v>231</v>
       </c>
-      <c r="M29" t="s" s="16">
+      <c r="M29" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N29" t="s" s="16">
+      <c r="N29" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P29" t="s" s="16">
+      <c r="P29" t="s" s="18">
         <v>232</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="s" s="16">
+      <c r="A30" t="s" s="18">
         <v>233</v>
       </c>
-      <c r="B30" t="s" s="16">
+      <c r="B30" t="s" s="18">
         <v>213</v>
       </c>
-      <c r="C30" t="s" s="16">
+      <c r="C30" t="s" s="18">
         <v>214</v>
       </c>
-      <c r="D30" t="s" s="16">
+      <c r="D30" t="s" s="18">
         <v>234</v>
       </c>
-      <c r="E30" t="s" s="16">
+      <c r="E30" t="s" s="18">
         <v>27</v>
       </c>
-      <c r="F30" t="s" s="16">
+      <c r="F30" t="s" s="18">
         <v>216</v>
       </c>
-      <c r="G30" t="s" s="16">
+      <c r="G30" t="s" s="18">
         <v>235</v>
       </c>
-      <c r="H30" t="s" s="16">
+      <c r="H30" t="s" s="18">
         <v>236</v>
       </c>
-      <c r="I30" t="s" s="16">
+      <c r="I30" t="s" s="18">
         <v>237</v>
       </c>
-      <c r="J30" t="s" s="16">
+      <c r="J30" t="s" s="18">
         <v>238</v>
       </c>
-      <c r="K30" t="s" s="16">
+      <c r="K30" t="s" s="18">
         <v>239</v>
       </c>
-      <c r="L30" t="s" s="16">
+      <c r="L30" t="s" s="18">
         <v>240</v>
       </c>
-      <c r="M30" t="s" s="16">
+      <c r="M30" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N30" t="s" s="16">
+      <c r="N30" t="s" s="18">
         <v>344</v>
       </c>
-      <c r="P30" t="s" s="16">
+      <c r="P30" t="s" s="18">
         <v>242</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="s" s="16">
+      <c r="A31" t="s" s="18">
         <v>243</v>
       </c>
-      <c r="B31" t="s" s="16">
+      <c r="B31" t="s" s="18">
         <v>213</v>
       </c>
-      <c r="C31" t="s" s="16">
+      <c r="C31" t="s" s="18">
         <v>244</v>
       </c>
-      <c r="D31" t="s" s="16">
+      <c r="D31" t="s" s="18">
         <v>245</v>
       </c>
-      <c r="E31" t="s" s="16">
+      <c r="E31" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F31" t="s" s="16">
+      <c r="F31" t="s" s="18">
         <v>216</v>
       </c>
-      <c r="G31" t="s" s="16">
+      <c r="G31" t="s" s="18">
         <v>18</v>
       </c>
-      <c r="H31" t="s" s="16">
+      <c r="H31" t="s" s="18">
         <v>246</v>
       </c>
-      <c r="I31" t="s" s="16">
+      <c r="I31" t="s" s="18">
         <v>247</v>
       </c>
-      <c r="J31" t="s" s="16">
+      <c r="J31" t="s" s="18">
         <v>248</v>
       </c>
-      <c r="K31" t="s" s="16">
+      <c r="K31" t="s" s="18">
         <v>221</v>
       </c>
-      <c r="L31" t="s" s="16">
+      <c r="L31" t="s" s="18">
         <v>249</v>
       </c>
-      <c r="M31" t="s" s="16">
+      <c r="M31" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N31" t="s" s="16">
+      <c r="N31" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P31" t="s" s="16">
+      <c r="P31" t="s" s="18">
         <v>250</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="s" s="16">
+      <c r="A32" t="s" s="18">
         <v>251</v>
       </c>
-      <c r="B32" t="s" s="16">
+      <c r="B32" t="s" s="18">
         <v>213</v>
       </c>
-      <c r="C32" t="s" s="16">
+      <c r="C32" t="s" s="18">
         <v>244</v>
       </c>
-      <c r="D32" t="s" s="16">
+      <c r="D32" t="s" s="18">
         <v>252</v>
       </c>
-      <c r="E32" t="s" s="16">
+      <c r="E32" t="s" s="18">
         <v>27</v>
       </c>
-      <c r="F32" t="s" s="16">
+      <c r="F32" t="s" s="18">
         <v>216</v>
       </c>
-      <c r="G32" t="s" s="16">
+      <c r="G32" t="s" s="18">
         <v>18</v>
       </c>
-      <c r="H32" t="s" s="16">
+      <c r="H32" t="s" s="18">
         <v>253</v>
       </c>
-      <c r="I32" t="s" s="16">
+      <c r="I32" t="s" s="18">
         <v>254</v>
       </c>
-      <c r="J32" t="s" s="16">
+      <c r="J32" t="s" s="18">
         <v>255</v>
       </c>
-      <c r="K32" t="s" s="16">
+      <c r="K32" t="s" s="18">
         <v>230</v>
       </c>
-      <c r="L32" t="s" s="16">
+      <c r="L32" t="s" s="18">
         <v>256</v>
       </c>
-      <c r="M32" t="s" s="16">
+      <c r="M32" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N32" t="s" s="16">
+      <c r="N32" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P32" t="s" s="16">
+      <c r="P32" t="s" s="18">
         <v>13</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="s" s="16">
+      <c r="A33" t="s" s="18">
         <v>257</v>
       </c>
-      <c r="B33" t="s" s="16">
+      <c r="B33" t="s" s="18">
         <v>213</v>
       </c>
-      <c r="C33" t="s" s="16">
+      <c r="C33" t="s" s="18">
         <v>214</v>
       </c>
-      <c r="D33" t="s" s="16">
+      <c r="D33" t="s" s="18">
         <v>350</v>
       </c>
-      <c r="E33" t="s" s="16">
+      <c r="E33" t="s" s="18">
         <v>27</v>
       </c>
-      <c r="F33" t="s" s="16">
+      <c r="F33" t="s" s="18">
         <v>216</v>
       </c>
-      <c r="G33" t="s" s="16">
+      <c r="G33" t="s" s="18">
         <v>259</v>
       </c>
-      <c r="H33" t="s" s="16">
+      <c r="H33" t="s" s="18">
         <v>351</v>
       </c>
-      <c r="I33" t="s" s="16">
+      <c r="I33" t="s" s="18">
         <v>352</v>
       </c>
-      <c r="J33" t="s" s="16">
+      <c r="J33" t="s" s="18">
         <v>353</v>
       </c>
-      <c r="K33" t="s" s="16">
+      <c r="K33" t="s" s="18">
         <v>230</v>
       </c>
-      <c r="L33" t="s" s="16">
+      <c r="L33" t="s" s="18">
         <v>354</v>
       </c>
-      <c r="M33" t="s" s="16">
+      <c r="M33" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N33" t="s" s="16">
+      <c r="N33" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P33" t="s" s="16">
+      <c r="P33" t="s" s="18">
         <v>355</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="s" s="16">
+      <c r="A34" t="s" s="18">
         <v>265</v>
       </c>
-      <c r="B34" t="s" s="16">
+      <c r="B34" t="s" s="18">
         <v>266</v>
       </c>
-      <c r="C34" t="s" s="16">
+      <c r="C34" t="s" s="18">
         <v>121</v>
       </c>
-      <c r="D34" t="s" s="16">
+      <c r="D34" t="s" s="18">
         <v>267</v>
       </c>
-      <c r="E34" t="s" s="16">
+      <c r="E34" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="F34" t="s" s="16">
+      <c r="F34" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="G34" t="s" s="16">
+      <c r="G34" t="s" s="18">
         <v>268</v>
       </c>
-      <c r="H34" t="s" s="16">
+      <c r="H34" t="s" s="18">
         <v>269</v>
       </c>
-      <c r="I34" t="s" s="16">
+      <c r="I34" t="s" s="18">
         <v>270</v>
       </c>
-      <c r="J34" t="s" s="16">
+      <c r="J34" t="s" s="18">
         <v>271</v>
       </c>
-      <c r="K34" t="s" s="16">
+      <c r="K34" t="s" s="18">
         <v>272</v>
       </c>
-      <c r="L34" t="s" s="16">
+      <c r="L34" t="s" s="18">
         <v>273</v>
       </c>
-      <c r="M34" t="s" s="16">
+      <c r="M34" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="N34" t="s" s="16">
+      <c r="N34" t="s" s="18">
         <v>343</v>
       </c>
-      <c r="P34" t="s" s="16">
+      <c r="P34" t="s" s="18">
         <v>274</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s" s="18">
+        <v>365</v>
+      </c>
+      <c r="B35" t="s" s="18">
+        <v>129</v>
+      </c>
+      <c r="C35" t="s" s="18">
+        <v>170</v>
+      </c>
+      <c r="D35" t="s" s="18">
+        <v>366</v>
+      </c>
+      <c r="E35" t="s" s="18">
+        <v>27</v>
+      </c>
+      <c r="F35" t="s" s="18">
+        <v>5</v>
+      </c>
+      <c r="G35" t="s" s="18">
+        <v>179</v>
+      </c>
+      <c r="H35" t="s" s="18">
+        <v>367</v>
+      </c>
+      <c r="I35" t="s" s="18">
+        <v>368</v>
+      </c>
+      <c r="J35" t="s" s="18">
+        <v>369</v>
+      </c>
+      <c r="K35" t="s" s="18">
+        <v>166</v>
+      </c>
+      <c r="L35" t="s" s="18">
+        <v>370</v>
+      </c>
+      <c r="M35" t="s" s="18">
+        <v>12</v>
+      </c>
+      <c r="N35" t="s" s="18">
+        <v>343</v>
+      </c>
+      <c r="P35" t="s" s="18">
+        <v>371</v>
       </c>
     </row>
   </sheetData>
@@ -3752,240 +3861,240 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="16">
+      <c r="A2" t="s" s="18">
         <v>275</v>
       </c>
-      <c r="B2" t="s" s="16">
+      <c r="B2" t="s" s="18">
         <v>2</v>
       </c>
-      <c r="C2" t="s" s="16">
+      <c r="C2" t="s" s="18">
         <v>0</v>
       </c>
-      <c r="D2" t="s" s="16">
+      <c r="D2" t="s" s="18">
         <v>276</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="16">
+      <c r="A3" t="s" s="18">
         <v>275</v>
       </c>
-      <c r="B3" t="s" s="16">
+      <c r="B3" t="s" s="18">
         <v>16</v>
       </c>
-      <c r="C3" t="s" s="16">
+      <c r="C3" t="s" s="18">
         <v>277</v>
       </c>
-      <c r="D3" t="s" s="16">
+      <c r="D3" t="s" s="18">
         <v>278</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s" s="16">
+      <c r="A4" t="s" s="18">
         <v>275</v>
       </c>
-      <c r="B4" t="s" s="16">
+      <c r="B4" t="s" s="18">
         <v>42</v>
       </c>
-      <c r="C4" t="s" s="16">
+      <c r="C4" t="s" s="18">
         <v>41</v>
       </c>
-      <c r="D4" t="s" s="16">
+      <c r="D4" t="s" s="18">
         <v>276</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s" s="16">
+      <c r="A5" t="s" s="18">
         <v>279</v>
       </c>
-      <c r="B5" t="s" s="16">
+      <c r="B5" t="s" s="18">
         <v>58</v>
       </c>
-      <c r="C5" t="s" s="16">
+      <c r="C5" t="s" s="18">
         <v>280</v>
       </c>
-      <c r="D5" t="s" s="16">
+      <c r="D5" t="s" s="18">
         <v>281</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s" s="16">
+      <c r="A6" t="s" s="18">
         <v>279</v>
       </c>
-      <c r="B6" t="s" s="16">
+      <c r="B6" t="s" s="18">
         <v>76</v>
       </c>
-      <c r="C6" t="s" s="16">
+      <c r="C6" t="s" s="18">
         <v>282</v>
       </c>
-      <c r="D6" t="s" s="16">
+      <c r="D6" t="s" s="18">
         <v>283</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s" s="16">
+      <c r="A7" t="s" s="18">
         <v>279</v>
       </c>
-      <c r="B7" t="s" s="16">
+      <c r="B7" t="s" s="18">
         <v>99</v>
       </c>
-      <c r="C7" t="s" s="16">
+      <c r="C7" t="s" s="18">
         <v>98</v>
       </c>
-      <c r="D7" t="s" s="16">
+      <c r="D7" t="s" s="18">
         <v>276</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="s" s="16">
+      <c r="A8" t="s" s="18">
         <v>284</v>
       </c>
-      <c r="B8" t="s" s="16">
+      <c r="B8" t="s" s="18">
         <v>130</v>
       </c>
-      <c r="C8" t="s" s="16">
+      <c r="C8" t="s" s="18">
         <v>285</v>
       </c>
-      <c r="D8" t="s" s="16">
+      <c r="D8" t="s" s="18">
         <v>276</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="s" s="16">
+      <c r="A9" t="s" s="18">
         <v>284</v>
       </c>
-      <c r="B9" t="s" s="16">
+      <c r="B9" t="s" s="18">
         <v>139</v>
       </c>
-      <c r="C9" t="s" s="16">
+      <c r="C9" t="s" s="18">
         <v>286</v>
       </c>
-      <c r="D9" t="s" s="16">
+      <c r="D9" t="s" s="18">
         <v>278</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="s" s="16">
+      <c r="A10" t="s" s="18">
         <v>284</v>
       </c>
-      <c r="B10" t="s" s="16">
+      <c r="B10" t="s" s="18">
         <v>170</v>
       </c>
-      <c r="C10" t="s" s="16">
-        <v>287</v>
-      </c>
-      <c r="D10" t="s" s="16">
+      <c r="C10" t="s" s="18">
+        <v>376</v>
+      </c>
+      <c r="D10" t="s" s="18">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="18">
+        <v>289</v>
+      </c>
+      <c r="B11" t="s" s="18">
+        <v>290</v>
+      </c>
+      <c r="C11" t="s" s="18">
+        <v>291</v>
+      </c>
+      <c r="D11" t="s" s="18">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="18">
+        <v>289</v>
+      </c>
+      <c r="B12" t="s" s="18">
+        <v>292</v>
+      </c>
+      <c r="C12" t="s" s="18">
+        <v>293</v>
+      </c>
+      <c r="D12" t="s" s="18">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="18">
+        <v>289</v>
+      </c>
+      <c r="B13" t="s" s="18">
+        <v>294</v>
+      </c>
+      <c r="C13" t="s" s="18">
+        <v>295</v>
+      </c>
+      <c r="D13" t="s" s="18">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="18">
+        <v>289</v>
+      </c>
+      <c r="B14" t="s" s="18">
+        <v>297</v>
+      </c>
+      <c r="C14" t="s" s="18">
+        <v>298</v>
+      </c>
+      <c r="D14" t="s" s="18">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="18">
+        <v>299</v>
+      </c>
+      <c r="B15" t="s" s="18">
+        <v>300</v>
+      </c>
+      <c r="C15" t="s" s="18">
+        <v>301</v>
+      </c>
+      <c r="D15" t="s" s="18">
         <v>288</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="s" s="16">
-        <v>289</v>
-      </c>
-      <c r="B11" t="s" s="16">
-        <v>290</v>
-      </c>
-      <c r="C11" t="s" s="16">
-        <v>291</v>
-      </c>
-      <c r="D11" t="s" s="16">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="16">
-        <v>289</v>
-      </c>
-      <c r="B12" t="s" s="16">
-        <v>292</v>
-      </c>
-      <c r="C12" t="s" s="16">
-        <v>293</v>
-      </c>
-      <c r="D12" t="s" s="16">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s" s="16">
-        <v>289</v>
-      </c>
-      <c r="B13" t="s" s="16">
-        <v>294</v>
-      </c>
-      <c r="C13" t="s" s="16">
-        <v>295</v>
-      </c>
-      <c r="D13" t="s" s="16">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s" s="16">
-        <v>289</v>
-      </c>
-      <c r="B14" t="s" s="16">
-        <v>297</v>
-      </c>
-      <c r="C14" t="s" s="16">
-        <v>298</v>
-      </c>
-      <c r="D14" t="s" s="16">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s" s="16">
+    <row r="16">
+      <c r="A16" t="s" s="18">
         <v>299</v>
       </c>
-      <c r="B15" t="s" s="16">
-        <v>300</v>
-      </c>
-      <c r="C15" t="s" s="16">
-        <v>301</v>
-      </c>
-      <c r="D15" t="s" s="16">
+      <c r="B16" t="s" s="18">
+        <v>302</v>
+      </c>
+      <c r="C16" t="s" s="18">
+        <v>303</v>
+      </c>
+      <c r="D16" t="s" s="18">
         <v>288</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="s" s="16">
+    <row r="17">
+      <c r="A17" t="s" s="18">
         <v>299</v>
       </c>
-      <c r="B16" t="s" s="16">
-        <v>302</v>
-      </c>
-      <c r="C16" t="s" s="16">
-        <v>303</v>
-      </c>
-      <c r="D16" t="s" s="16">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s" s="16">
+      <c r="B17" t="s" s="18">
+        <v>304</v>
+      </c>
+      <c r="C17" t="s" s="18">
+        <v>305</v>
+      </c>
+      <c r="D17" t="s" s="18">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="18">
         <v>299</v>
       </c>
-      <c r="B17" t="s" s="16">
-        <v>304</v>
-      </c>
-      <c r="C17" t="s" s="16">
-        <v>305</v>
-      </c>
-      <c r="D17" t="s" s="16">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s" s="16">
-        <v>299</v>
-      </c>
-      <c r="B18" t="s" s="16">
+      <c r="B18" t="s" s="18">
         <v>306</v>
       </c>
-      <c r="C18" t="s" s="16">
+      <c r="C18" t="s" s="18">
         <v>307</v>
       </c>
-      <c r="D18" t="s" s="16">
+      <c r="D18" t="s" s="18">
         <v>296</v>
       </c>
     </row>
@@ -4000,7 +4109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="8.0"/>
@@ -4032,199 +4141,213 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="16">
+      <c r="A2" t="s" s="18">
         <v>308</v>
       </c>
-      <c r="B2" t="s" s="16">
+      <c r="B2" t="s" s="18">
         <v>309</v>
       </c>
-      <c r="C2" t="s" s="16">
+      <c r="C2" t="s" s="18">
         <v>310</v>
       </c>
-      <c r="D2" t="s" s="16">
+      <c r="D2" t="s" s="18">
         <v>311</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="16">
+      <c r="A3" t="s" s="18">
         <v>312</v>
       </c>
-      <c r="B3" t="s" s="16">
+      <c r="B3" t="s" s="18">
         <v>309</v>
       </c>
-      <c r="C3" t="s" s="16">
+      <c r="C3" t="s" s="18">
         <v>313</v>
       </c>
-      <c r="D3" t="s" s="16">
+      <c r="D3" t="s" s="18">
         <v>314</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s" s="16">
+      <c r="A4" t="s" s="18">
         <v>315</v>
       </c>
-      <c r="B4" t="s" s="16">
+      <c r="B4" t="s" s="18">
         <v>309</v>
       </c>
-      <c r="C4" t="s" s="16">
+      <c r="C4" t="s" s="18">
         <v>316</v>
       </c>
-      <c r="D4" t="s" s="16">
+      <c r="D4" t="s" s="18">
         <v>317</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s" s="16">
+      <c r="A5" t="s" s="18">
         <v>318</v>
       </c>
-      <c r="B5" t="s" s="16">
+      <c r="B5" t="s" s="18">
         <v>319</v>
       </c>
-      <c r="C5" t="s" s="16">
+      <c r="C5" t="s" s="18">
         <v>320</v>
       </c>
-      <c r="D5" t="s" s="16">
+      <c r="D5" t="s" s="18">
         <v>321</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s" s="16">
+      <c r="A6" t="s" s="18">
         <v>322</v>
       </c>
-      <c r="B6" t="s" s="16">
+      <c r="B6" t="s" s="18">
         <v>323</v>
       </c>
-      <c r="C6" t="s" s="16">
+      <c r="C6" t="s" s="18">
         <v>324</v>
       </c>
-      <c r="D6" t="s" s="16">
+      <c r="D6" t="s" s="18">
         <v>233</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s" s="16">
+      <c r="A7" t="s" s="18">
         <v>325</v>
       </c>
-      <c r="B7" t="s" s="16">
+      <c r="B7" t="s" s="18">
         <v>319</v>
       </c>
-      <c r="C7" t="s" s="16">
+      <c r="C7" t="s" s="18">
         <v>326</v>
       </c>
-      <c r="D7" t="s" s="16">
+      <c r="D7" t="s" s="18">
         <v>327</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="s" s="16">
+      <c r="A8" t="s" s="18">
         <v>328</v>
       </c>
-      <c r="B8" t="s" s="16">
+      <c r="B8" t="s" s="18">
         <v>319</v>
       </c>
-      <c r="C8" t="s" s="16">
+      <c r="C8" t="s" s="18">
         <v>329</v>
       </c>
-      <c r="D8" t="s" s="16">
+      <c r="D8" t="s" s="18">
         <v>113</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="s" s="16">
+      <c r="A9" t="s" s="18">
         <v>330</v>
       </c>
-      <c r="B9" t="s" s="16">
+      <c r="B9" t="s" s="18">
         <v>319</v>
       </c>
-      <c r="C9" t="s" s="16">
+      <c r="C9" t="s" s="18">
         <v>331</v>
       </c>
-      <c r="D9" t="s" s="16">
+      <c r="D9" t="s" s="18">
         <v>257</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="s" s="16">
+      <c r="A10" t="s" s="18">
         <v>332</v>
       </c>
-      <c r="B10" t="s" s="16">
+      <c r="B10" t="s" s="18">
         <v>319</v>
       </c>
-      <c r="C10" t="s" s="16">
+      <c r="C10" t="s" s="18">
         <v>333</v>
       </c>
-      <c r="D10" t="s" s="16">
+      <c r="D10" t="s" s="18">
         <v>67</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="s" s="16">
+      <c r="A11" t="s" s="18">
         <v>334</v>
       </c>
-      <c r="B11" t="s" s="16">
+      <c r="B11" t="s" s="18">
         <v>319</v>
       </c>
-      <c r="C11" t="s" s="16">
+      <c r="C11" t="s" s="18">
         <v>335</v>
       </c>
-      <c r="D11" t="s" s="16">
+      <c r="D11" t="s" s="18">
         <v>336</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="s" s="16">
+      <c r="A12" t="s" s="18">
         <v>337</v>
       </c>
-      <c r="B12" t="s" s="16">
+      <c r="B12" t="s" s="18">
         <v>338</v>
       </c>
-      <c r="C12" t="s" s="16">
+      <c r="C12" t="s" s="18">
         <v>339</v>
       </c>
-      <c r="D12" t="s" s="16">
+      <c r="D12" t="s" s="18">
         <v>233</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="s" s="16">
+      <c r="A13" t="s" s="18">
         <v>340</v>
       </c>
-      <c r="B13" t="s" s="16">
+      <c r="B13" t="s" s="18">
         <v>338</v>
       </c>
-      <c r="C13" t="s" s="16">
+      <c r="C13" t="s" s="18">
         <v>341</v>
       </c>
-      <c r="D13" t="s" s="16">
+      <c r="D13" t="s" s="18">
         <v>342</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="s" s="16">
+      <c r="A14" t="s" s="18">
         <v>348</v>
       </c>
-      <c r="B14" t="s" s="16">
+      <c r="B14" t="s" s="18">
         <v>319</v>
       </c>
-      <c r="C14" t="s" s="16">
+      <c r="C14" t="s" s="18">
         <v>349</v>
       </c>
-      <c r="D14" t="s" s="16">
+      <c r="D14" t="s" s="18">
         <v>15</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="s" s="16">
+      <c r="A15" t="s" s="18">
         <v>356</v>
       </c>
-      <c r="B15" t="s" s="16">
+      <c r="B15" t="s" s="18">
         <v>319</v>
       </c>
-      <c r="C15" t="s" s="16">
+      <c r="C15" t="s" s="18">
         <v>357</v>
       </c>
-      <c r="D15" t="s" s="16">
+      <c r="D15" t="s" s="18">
         <v>257</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="18">
+        <v>372</v>
+      </c>
+      <c r="B16" t="s" s="18">
+        <v>319</v>
+      </c>
+      <c r="C16" t="s" s="18">
+        <v>373</v>
+      </c>
+      <c r="D16" t="s" s="18">
+        <v>374</v>
       </c>
     </row>
   </sheetData>

</xml_diff>